<commit_message>
Data. collect_predictions.py manual para verificar su correcto funcionamiento.
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
+++ b/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O47"/>
+  <dimension ref="A1:O57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1127,2230 +1127,2855 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>tYjCfe2E</t>
+          <t>8j9FTL56</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>45514.45833333334</v>
+        <v>45528.35416666666</v>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
+          <t xml:space="preserve">amex stadium
+  brighton </t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>31876</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2XrRecc3</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>brighton</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>ppjDR086</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>manchester utd</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>48</v>
+      </c>
+      <c r="K12" t="n">
+        <v>481</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>U5cORazJ</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>45528.45833333334</v>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">selhurst park
+  london </t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>25486</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>AovF1Mia</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>crystal palace</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Cxq57r8g</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>west ham</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>48</v>
+      </c>
+      <c r="K13" t="n">
+        <v>481</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>dCkAk3SP</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>45528.45833333334</v>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">craven cottage
+  london </t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>26600</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>69ZiU2Om</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>fulham</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>KrrdAMyI</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>leicester</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>48</v>
+      </c>
+      <c r="K14" t="n">
+        <v>481</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>lAUlrLKa</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>45528.45833333334</v>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">etihad stadium
+  manchester </t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>55097</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Wtn9Stg0</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>manchester city</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>thqhB2MB</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>ipswich</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>48</v>
+      </c>
+      <c r="K15" t="n">
+        <v>481</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>fNaktakC</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>45528.45833333334</v>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">st  mary s stadium
+  southampton </t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>32384</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>WdKOwxDM</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>southampton</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>UsushcZr</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>nottingham</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>48</v>
+      </c>
+      <c r="K16" t="n">
+        <v>481</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>2m3cvwKO</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>45528.45833333334</v>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tottenham hotspur stadium
+  london </t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>62850</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>UDg08Ohm</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>tottenham</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>KluSTr9s</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>everton</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>48</v>
+      </c>
+      <c r="K17" t="n">
+        <v>481</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>2g67Vsyf</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>45528.5625</v>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">villa park
+  birmingham </t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>42789</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>W00wmLO0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>aston villa</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>hA1Zm19f</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>arsenal</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>48</v>
+      </c>
+      <c r="K18" t="n">
+        <v>481</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>6RCbX36s</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>45529.41666666666</v>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vitality stadium
+  bournemouth </t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>11307</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>OtpNdwrc</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>bournemouth</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>p6ahwuwJ</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>newcastle</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>48</v>
+      </c>
+      <c r="K19" t="n">
+        <v>481</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>61T7bt5t</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>45529.41666666666</v>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">molineux stadium
+  wolverhampton </t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>31750</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>j3Azpf5d</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>wolves</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>4fGZN2oK</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>chelsea</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>48</v>
+      </c>
+      <c r="K20" t="n">
+        <v>481</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>GdWtpsjm</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>45529.52083333334</v>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">anfield
+  liverpool </t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>61276</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>lId4TMwf</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>liverpool</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>xYe7DwID</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>brentford</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>48</v>
+      </c>
+      <c r="K21" t="n">
+        <v>481</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>tYjCfe2E</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>45514.45833333334</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gillett j 
+  aus </t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
           <t xml:space="preserve">wembley stadium
   london </t>
         </is>
       </c>
-      <c r="E12" t="n">
+      <c r="E22" t="n">
         <v>90000</v>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Wtn9Stg0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>manchester city</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
         <is>
           <t>ppjDR086</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>manchester utd</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Wtn9Stg0</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>manchester city</t>
-        </is>
-      </c>
-      <c r="J12" t="n">
-        <v>48</v>
-      </c>
-      <c r="K12" t="n">
+      <c r="J22" t="n">
+        <v>48</v>
+      </c>
+      <c r="K22" t="n">
         <v>482</v>
       </c>
-      <c r="L12" t="n">
+      <c r="L22" t="n">
         <v>1</v>
       </c>
-      <c r="M12" t="n">
+      <c r="M22" t="n">
         <v>2024</v>
       </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
         <is>
           <t>fa community shield</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>OMDVg8x9</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B23" s="2" t="n">
         <v>45517.64583333334</v>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
         <is>
           <t xml:space="preserve">brunton park
   carlisle </t>
         </is>
       </c>
-      <c r="E13" t="n">
+      <c r="E23" t="n">
         <v>17949</v>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>dUzTIwSF</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>carlisle</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>hSUajdSS</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>stoke</t>
         </is>
       </c>
-      <c r="J13" t="n">
-        <v>48</v>
-      </c>
-      <c r="K13" t="n">
+      <c r="J23" t="n">
+        <v>48</v>
+      </c>
+      <c r="K23" t="n">
         <v>484</v>
       </c>
-      <c r="L13" t="n">
+      <c r="L23" t="n">
         <v>1</v>
       </c>
-      <c r="M13" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
+      <c r="M23" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
         <is>
           <t>jXcAnQUr</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B24" s="2" t="n">
         <v>45517.64583333334</v>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr">
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
         <is>
           <t xml:space="preserve">brisbane road
   london </t>
         </is>
       </c>
-      <c r="E14" t="n">
+      <c r="E24" t="n">
         <v>9271</v>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>KKyYcus9</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>leyton orient</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>ChwgcrNJ</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>newport</t>
         </is>
       </c>
-      <c r="J14" t="n">
-        <v>48</v>
-      </c>
-      <c r="K14" t="n">
+      <c r="J24" t="n">
+        <v>48</v>
+      </c>
+      <c r="K24" t="n">
         <v>484</v>
       </c>
-      <c r="L14" t="n">
+      <c r="L24" t="n">
         <v>1</v>
       </c>
-      <c r="M14" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
+      <c r="M24" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
         <is>
           <t>fRe0c20b</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B25" s="2" t="n">
         <v>45517.64583333334</v>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr">
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
         <is>
           <t xml:space="preserve">edgeley park
   stockport </t>
         </is>
       </c>
-      <c r="E15" t="n">
+      <c r="E25" t="n">
         <v>10841</v>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>IX6WjNvr</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>stockport county</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>6Nl8nagD</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>blackburn</t>
         </is>
       </c>
-      <c r="J15" t="n">
-        <v>48</v>
-      </c>
-      <c r="K15" t="n">
+      <c r="J25" t="n">
+        <v>48</v>
+      </c>
+      <c r="K25" t="n">
         <v>484</v>
       </c>
-      <c r="L15" t="n">
+      <c r="L25" t="n">
         <v>1</v>
       </c>
-      <c r="M15" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
+      <c r="M25" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
         <is>
           <t>CnnJp4ae</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B26" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr">
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
         <is>
           <t xml:space="preserve">holker street
   barrow in furness </t>
         </is>
       </c>
-      <c r="E16" t="n">
+      <c r="E26" t="n">
         <v>6500</v>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>KKJL7QXd</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>barrow</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>U3lM3y4e</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>port vale</t>
         </is>
       </c>
-      <c r="J16" t="n">
-        <v>48</v>
-      </c>
-      <c r="K16" t="n">
+      <c r="J26" t="n">
+        <v>48</v>
+      </c>
+      <c r="K26" t="n">
         <v>484</v>
       </c>
-      <c r="L16" t="n">
+      <c r="L26" t="n">
         <v>1</v>
       </c>
-      <c r="M16" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
+      <c r="M26" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t>bw1zAKS6</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n">
+      <c r="B27" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr">
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
         <is>
           <t xml:space="preserve">toughsheet community stadium
   bolton </t>
         </is>
       </c>
-      <c r="E17" t="n">
+      <c r="E27" t="n">
         <v>28723</v>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>Or1bBrWD</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>bolton</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>t6G9wMZN</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>mansfield</t>
         </is>
       </c>
-      <c r="J17" t="n">
-        <v>48</v>
-      </c>
-      <c r="K17" t="n">
+      <c r="J27" t="n">
+        <v>48</v>
+      </c>
+      <c r="K27" t="n">
         <v>484</v>
       </c>
-      <c r="L17" t="n">
+      <c r="L27" t="n">
         <v>1</v>
       </c>
-      <c r="M17" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
+      <c r="M27" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
         <is>
           <t>GINCsvmn</t>
         </is>
       </c>
-      <c r="B18" s="2" t="n">
+      <c r="B28" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr">
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
         <is>
           <t xml:space="preserve">ashton gate stadium
   bristol </t>
         </is>
       </c>
-      <c r="E18" t="n">
+      <c r="E28" t="n">
         <v>27000</v>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>MahqU27I</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>bristol city</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>GOvB22xg</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>coventry</t>
         </is>
       </c>
-      <c r="J18" t="n">
-        <v>48</v>
-      </c>
-      <c r="K18" t="n">
+      <c r="J28" t="n">
+        <v>48</v>
+      </c>
+      <c r="K28" t="n">
         <v>484</v>
       </c>
-      <c r="L18" t="n">
+      <c r="L28" t="n">
         <v>1</v>
       </c>
-      <c r="M18" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
+      <c r="M28" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
         <is>
           <t>x6klsVh3</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B29" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr">
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
         <is>
           <t xml:space="preserve">hayes lane
   london </t>
         </is>
       </c>
-      <c r="E19" t="n">
+      <c r="E29" t="n">
         <v>5000</v>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>Opdcd08Q</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>bromley</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>4KREuF43</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>afc wimbledon</t>
         </is>
       </c>
-      <c r="J19" t="n">
-        <v>48</v>
-      </c>
-      <c r="K19" t="n">
+      <c r="J29" t="n">
+        <v>48</v>
+      </c>
+      <c r="K29" t="n">
         <v>484</v>
       </c>
-      <c r="L19" t="n">
+      <c r="L29" t="n">
         <v>1</v>
       </c>
-      <c r="M19" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
+      <c r="M29" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
         <is>
           <t>b3pRrrU7</t>
         </is>
       </c>
-      <c r="B20" s="2" t="n">
+      <c r="B30" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr">
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
         <is>
           <t xml:space="preserve">pirelli stadium
   burton upon trent </t>
         </is>
       </c>
-      <c r="E20" t="n">
+      <c r="E30" t="n">
         <v>6912</v>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>nwCtJaJT</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>burton</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>8EFIJthC</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>blackpool</t>
         </is>
       </c>
-      <c r="J20" t="n">
-        <v>48</v>
-      </c>
-      <c r="K20" t="n">
+      <c r="J30" t="n">
+        <v>48</v>
+      </c>
+      <c r="K30" t="n">
         <v>484</v>
       </c>
-      <c r="L20" t="n">
+      <c r="L30" t="n">
         <v>1</v>
       </c>
-      <c r="M20" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
+      <c r="M30" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
         <is>
           <t>WfkfPdXH</t>
         </is>
       </c>
-      <c r="B21" s="2" t="n">
+      <c r="B31" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr">
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
         <is>
           <t xml:space="preserve">abbey stadium
   cambridge </t>
         </is>
       </c>
-      <c r="E21" t="n">
+      <c r="E31" t="n">
         <v>7937</v>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>lnb8EJRp</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>cambridge utd</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>lrMHUHDc</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>qpr</t>
         </is>
       </c>
-      <c r="J21" t="n">
-        <v>48</v>
-      </c>
-      <c r="K21" t="n">
+      <c r="J31" t="n">
+        <v>48</v>
+      </c>
+      <c r="K31" t="n">
         <v>484</v>
       </c>
-      <c r="L21" t="n">
+      <c r="L31" t="n">
         <v>1</v>
       </c>
-      <c r="M21" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
+      <c r="M31" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
         <is>
           <t>SMr3Nz2U</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n">
+      <c r="B32" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr">
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
         <is>
           <t xml:space="preserve">cardiff city stadium
   cardiff </t>
         </is>
       </c>
-      <c r="E22" t="n">
+      <c r="E32" t="n">
         <v>33280</v>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>hO8wh6aP</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>cardiff</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>GILi6JC9</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>bristol rovers</t>
         </is>
       </c>
-      <c r="J22" t="n">
-        <v>48</v>
-      </c>
-      <c r="K22" t="n">
+      <c r="J32" t="n">
+        <v>48</v>
+      </c>
+      <c r="K32" t="n">
         <v>484</v>
       </c>
-      <c r="L22" t="n">
+      <c r="L32" t="n">
         <v>1</v>
       </c>
-      <c r="M22" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
+      <c r="M32" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
         <is>
           <t>xYBLuIHb</t>
         </is>
       </c>
-      <c r="B23" s="2" t="n">
+      <c r="B33" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr">
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
         <is>
           <t xml:space="preserve">the valley
   london </t>
         </is>
       </c>
-      <c r="E23" t="n">
+      <c r="E33" t="n">
         <v>27111</v>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>fXf5mQ7t</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>charlton</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>SWk4muv7</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>birmingham</t>
         </is>
       </c>
-      <c r="J23" t="n">
-        <v>48</v>
-      </c>
-      <c r="K23" t="n">
+      <c r="J33" t="n">
+        <v>48</v>
+      </c>
+      <c r="K33" t="n">
         <v>484</v>
       </c>
-      <c r="L23" t="n">
+      <c r="L33" t="n">
         <v>1</v>
       </c>
-      <c r="M23" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
+      <c r="M33" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
         <is>
           <t>6os5wmhS</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n">
+      <c r="B34" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr">
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
         <is>
           <t xml:space="preserve">colchester community stadium
   colchester </t>
         </is>
       </c>
-      <c r="E24" t="n">
+      <c r="E34" t="n">
         <v>10105</v>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>xYu73rNn</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>colchester</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>EmlVDpVP</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>reading</t>
         </is>
       </c>
-      <c r="J24" t="n">
-        <v>48</v>
-      </c>
-      <c r="K24" t="n">
+      <c r="J34" t="n">
+        <v>48</v>
+      </c>
+      <c r="K34" t="n">
         <v>484</v>
       </c>
-      <c r="L24" t="n">
+      <c r="L34" t="n">
         <v>1</v>
       </c>
-      <c r="M24" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
+      <c r="M34" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
         <is>
           <t>Kl7vhn7L</t>
         </is>
       </c>
-      <c r="B25" s="2" t="n">
+      <c r="B35" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr">
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
         <is>
           <t xml:space="preserve">the broadfield stadium
   crawley </t>
         </is>
       </c>
-      <c r="E25" t="n">
+      <c r="E35" t="n">
         <v>6134</v>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>QVmLl54o</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>crawley</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H35" t="inlineStr">
         <is>
           <t>xSloasB8</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>swindon</t>
         </is>
       </c>
-      <c r="J25" t="n">
-        <v>48</v>
-      </c>
-      <c r="K25" t="n">
+      <c r="J35" t="n">
+        <v>48</v>
+      </c>
+      <c r="K35" t="n">
         <v>484</v>
       </c>
-      <c r="L25" t="n">
+      <c r="L35" t="n">
         <v>1</v>
       </c>
-      <c r="M25" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
+      <c r="M35" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="1" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
         <is>
           <t>nw6fJO5K</t>
         </is>
       </c>
-      <c r="B26" s="2" t="n">
+      <c r="B36" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr">
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
         <is>
           <t xml:space="preserve">pride park
   derby </t>
         </is>
       </c>
-      <c r="E26" t="n">
+      <c r="E36" t="n">
         <v>33597</v>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>Iug0YO0Q</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>derby</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H36" t="inlineStr">
         <is>
           <t>dQIMIN5n</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>chesterfield</t>
         </is>
       </c>
-      <c r="J26" t="n">
-        <v>48</v>
-      </c>
-      <c r="K26" t="n">
+      <c r="J36" t="n">
+        <v>48</v>
+      </c>
+      <c r="K36" t="n">
         <v>484</v>
       </c>
-      <c r="L26" t="n">
+      <c r="L36" t="n">
         <v>1</v>
       </c>
-      <c r="M26" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
+      <c r="M36" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
         <is>
           <t>bHPacsq1</t>
         </is>
       </c>
-      <c r="B27" s="2" t="n">
+      <c r="B37" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr">
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
         <is>
           <t xml:space="preserve">highbury stadium
   fleetwood </t>
         </is>
       </c>
-      <c r="E27" t="n">
+      <c r="E37" t="n">
         <v>5327</v>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>tCZ3D68d</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>fleetwood</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>CCBWpzjj</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>west brom</t>
         </is>
       </c>
-      <c r="J27" t="n">
-        <v>48</v>
-      </c>
-      <c r="K27" t="n">
+      <c r="J37" t="n">
+        <v>48</v>
+      </c>
+      <c r="K37" t="n">
         <v>484</v>
       </c>
-      <c r="L27" t="n">
+      <c r="L37" t="n">
         <v>1</v>
       </c>
-      <c r="M27" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
+      <c r="M37" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="1" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
         <is>
           <t>MwmHgKaN</t>
         </is>
       </c>
-      <c r="B28" s="2" t="n">
+      <c r="B38" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr">
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
         <is>
           <t xml:space="preserve">blundell park
   cleethorpes </t>
         </is>
       </c>
-      <c r="E28" t="n">
+      <c r="E38" t="n">
         <v>9052</v>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>OEaiS3za</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>grimsby</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>bsc3EJ27</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>bradford city</t>
         </is>
       </c>
-      <c r="J28" t="n">
-        <v>48</v>
-      </c>
-      <c r="K28" t="n">
+      <c r="J38" t="n">
+        <v>48</v>
+      </c>
+      <c r="K38" t="n">
         <v>484</v>
       </c>
-      <c r="L28" t="n">
+      <c r="L38" t="n">
         <v>1</v>
       </c>
-      <c r="M28" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
+      <c r="M38" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="1" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr">
         <is>
           <t>lQl9etVA</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n">
+      <c r="B39" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr">
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
         <is>
           <t xml:space="preserve">john smith s stadium
   huddersfield </t>
         </is>
       </c>
-      <c r="E29" t="n">
+      <c r="E39" t="n">
         <v>24121</v>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>xxxpBZl2</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>huddersfield</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>zmKRcPKu</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>morecambe</t>
         </is>
       </c>
-      <c r="J29" t="n">
-        <v>48</v>
-      </c>
-      <c r="K29" t="n">
+      <c r="J39" t="n">
+        <v>48</v>
+      </c>
+      <c r="K39" t="n">
         <v>484</v>
       </c>
-      <c r="L29" t="n">
+      <c r="L39" t="n">
         <v>1</v>
       </c>
-      <c r="M29" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O29" t="inlineStr">
+      <c r="M39" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="1" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr">
         <is>
           <t>KWD8eLDD</t>
         </is>
       </c>
-      <c r="B30" s="2" t="n">
+      <c r="B40" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr">
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr">
         <is>
           <t xml:space="preserve">lner stadium
   lincoln </t>
         </is>
       </c>
-      <c r="E30" t="n">
+      <c r="E40" t="n">
         <v>10669</v>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>hrHTRs5B</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G40" t="inlineStr">
         <is>
           <t>lincoln</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>CQv5qrFt</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>harrogate</t>
         </is>
       </c>
-      <c r="J30" t="n">
-        <v>48</v>
-      </c>
-      <c r="K30" t="n">
+      <c r="J40" t="n">
+        <v>48</v>
+      </c>
+      <c r="K40" t="n">
         <v>484</v>
       </c>
-      <c r="L30" t="n">
+      <c r="L40" t="n">
         <v>1</v>
       </c>
-      <c r="M30" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr">
+      <c r="M40" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="1" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
         <is>
           <t>xUXzYQFk</t>
         </is>
       </c>
-      <c r="B31" s="2" t="n">
+      <c r="B41" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr">
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr">
         <is>
           <t xml:space="preserve">sixfields stadium
   northampton </t>
         </is>
       </c>
-      <c r="E31" t="n">
+      <c r="E41" t="n">
         <v>7798</v>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>l4P6dwRR</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G41" t="inlineStr">
         <is>
           <t>northampton</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="H41" t="inlineStr">
         <is>
           <t>hl2V5JIl</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>wycombe</t>
         </is>
       </c>
-      <c r="J31" t="n">
-        <v>48</v>
-      </c>
-      <c r="K31" t="n">
+      <c r="J41" t="n">
+        <v>48</v>
+      </c>
+      <c r="K41" t="n">
         <v>484</v>
       </c>
-      <c r="L31" t="n">
+      <c r="L41" t="n">
         <v>1</v>
       </c>
-      <c r="M31" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr">
+      <c r="M41" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="1" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
         <is>
           <t>CCV9JR0d</t>
         </is>
       </c>
-      <c r="B32" s="2" t="n">
+      <c r="B42" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr">
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
         <is>
           <t xml:space="preserve">carrow road
   norwich </t>
         </is>
       </c>
-      <c r="E32" t="n">
+      <c r="E42" t="n">
         <v>27137</v>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>Qo6off6p</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G42" t="inlineStr">
         <is>
           <t>norwich</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="H42" t="inlineStr">
         <is>
           <t>ANwyQM2M</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>stevenage</t>
         </is>
       </c>
-      <c r="J32" t="n">
-        <v>48</v>
-      </c>
-      <c r="K32" t="n">
+      <c r="J42" t="n">
+        <v>48</v>
+      </c>
+      <c r="K42" t="n">
         <v>484</v>
       </c>
-      <c r="L32" t="n">
+      <c r="L42" t="n">
         <v>1</v>
       </c>
-      <c r="M32" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr">
+      <c r="M42" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="1" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
         <is>
           <t>bsinRI25</t>
         </is>
       </c>
-      <c r="B33" s="2" t="n">
+      <c r="B43" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr">
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
         <is>
           <t xml:space="preserve">kassam stadium
   oxford </t>
         </is>
       </c>
-      <c r="E33" t="n">
+      <c r="E43" t="n">
         <v>12500</v>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>vgOBT43c</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G43" t="inlineStr">
         <is>
           <t>oxford utd</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>tWeI85kh</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>peterborough</t>
         </is>
       </c>
-      <c r="J33" t="n">
-        <v>48</v>
-      </c>
-      <c r="K33" t="n">
+      <c r="J43" t="n">
+        <v>48</v>
+      </c>
+      <c r="K43" t="n">
         <v>484</v>
       </c>
-      <c r="L33" t="n">
+      <c r="L43" t="n">
         <v>1</v>
       </c>
-      <c r="M33" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
+      <c r="M43" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="1" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
         <is>
           <t>GbaVU03t</t>
         </is>
       </c>
-      <c r="B34" s="2" t="n">
+      <c r="B44" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr">
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
         <is>
           <t xml:space="preserve">fratton park
   portsmouth </t>
         </is>
       </c>
-      <c r="E34" t="n">
+      <c r="E44" t="n">
         <v>21944</v>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>zckREQFJ</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G44" t="inlineStr">
         <is>
           <t>portsmouth</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H44" t="inlineStr">
         <is>
           <t>6uz2cJBL</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>millwall</t>
         </is>
       </c>
-      <c r="J34" t="n">
-        <v>48</v>
-      </c>
-      <c r="K34" t="n">
+      <c r="J44" t="n">
+        <v>48</v>
+      </c>
+      <c r="K44" t="n">
         <v>484</v>
       </c>
-      <c r="L34" t="n">
+      <c r="L44" t="n">
         <v>1</v>
       </c>
-      <c r="M34" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O34" t="inlineStr">
+      <c r="M44" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="1" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr">
         <is>
           <t>tOTmlbNp</t>
         </is>
       </c>
-      <c r="B35" s="2" t="n">
+      <c r="B45" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr">
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
         <is>
           <t xml:space="preserve">deepdale
   preston </t>
         </is>
       </c>
-      <c r="E35" t="n">
+      <c r="E45" t="n">
         <v>23408</v>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>x8IDVcbi</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G45" t="inlineStr">
         <is>
           <t>preston</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="H45" t="inlineStr">
         <is>
           <t>WSzc94ws</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>sunderland</t>
         </is>
       </c>
-      <c r="J35" t="n">
-        <v>48</v>
-      </c>
-      <c r="K35" t="n">
+      <c r="J45" t="n">
+        <v>48</v>
+      </c>
+      <c r="K45" t="n">
         <v>484</v>
       </c>
-      <c r="L35" t="n">
+      <c r="L45" t="n">
         <v>1</v>
       </c>
-      <c r="M35" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O35" t="inlineStr">
+      <c r="M45" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="1" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="1" t="inlineStr">
         <is>
           <t>nPQL4PjR</t>
         </is>
       </c>
-      <c r="B36" s="2" t="n">
+      <c r="B46" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr">
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr">
         <is>
           <t xml:space="preserve">aesseal new york stadium
   rotherham </t>
         </is>
       </c>
-      <c r="E36" t="n">
+      <c r="E46" t="n">
         <v>12021</v>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t>KMfM7P4b</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G46" t="inlineStr">
         <is>
           <t>rotherham</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="H46" t="inlineStr">
         <is>
           <t>YacqHHdS</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="I46" t="inlineStr">
         <is>
           <t>crewe</t>
         </is>
       </c>
-      <c r="J36" t="n">
-        <v>48</v>
-      </c>
-      <c r="K36" t="n">
+      <c r="J46" t="n">
+        <v>48</v>
+      </c>
+      <c r="K46" t="n">
         <v>484</v>
       </c>
-      <c r="L36" t="n">
+      <c r="L46" t="n">
         <v>1</v>
       </c>
-      <c r="M36" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O36" t="inlineStr">
+      <c r="M46" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="1" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr">
         <is>
           <t>pWhdu9NF</t>
         </is>
       </c>
-      <c r="B37" s="2" t="n">
+      <c r="B47" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr">
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
         <is>
           <t xml:space="preserve">peninsula stadium
   salford </t>
         </is>
       </c>
-      <c r="E37" t="n">
+      <c r="E47" t="n">
         <v>5108</v>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>W4AadhN3</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G47" t="inlineStr">
         <is>
           <t>salford</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="H47" t="inlineStr">
         <is>
           <t>hlzYDy5q</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>doncaster</t>
         </is>
       </c>
-      <c r="J37" t="n">
-        <v>48</v>
-      </c>
-      <c r="K37" t="n">
+      <c r="J47" t="n">
+        <v>48</v>
+      </c>
+      <c r="K47" t="n">
         <v>484</v>
       </c>
-      <c r="L37" t="n">
+      <c r="L47" t="n">
         <v>1</v>
       </c>
-      <c r="M37" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O37" t="inlineStr">
+      <c r="M47" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="1" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr">
         <is>
           <t>6NnRD2Ts</t>
         </is>
       </c>
-      <c r="B38" s="2" t="n">
+      <c r="B48" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr">
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr">
         <is>
           <t xml:space="preserve">the croud meadow
   shrewsbury </t>
         </is>
       </c>
-      <c r="E38" t="n">
+      <c r="E48" t="n">
         <v>9877</v>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F48" t="inlineStr">
         <is>
           <t>EqfQ6qK4</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="G48" t="inlineStr">
         <is>
           <t>shrewsbury</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="H48" t="inlineStr">
         <is>
           <t>EwJVdqzn</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="I48" t="inlineStr">
         <is>
           <t>notts co</t>
         </is>
       </c>
-      <c r="J38" t="n">
-        <v>48</v>
-      </c>
-      <c r="K38" t="n">
+      <c r="J48" t="n">
+        <v>48</v>
+      </c>
+      <c r="K48" t="n">
         <v>484</v>
       </c>
-      <c r="L38" t="n">
+      <c r="L48" t="n">
         <v>1</v>
       </c>
-      <c r="M38" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O38" t="inlineStr">
+      <c r="M48" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="1" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
         <is>
           <t>2FcwTvYh</t>
         </is>
       </c>
-      <c r="B39" s="2" t="n">
+      <c r="B49" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr">
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
         <is>
           <t xml:space="preserve">swansea com stadium
   swansea </t>
         </is>
       </c>
-      <c r="E39" t="n">
+      <c r="E49" t="n">
         <v>21088</v>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>K6xezbY7</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G49" t="inlineStr">
         <is>
           <t>swansea</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H49" t="inlineStr">
         <is>
           <t>WvZyDeKk</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>gillingham</t>
         </is>
       </c>
-      <c r="J39" t="n">
-        <v>48</v>
-      </c>
-      <c r="K39" t="n">
+      <c r="J49" t="n">
+        <v>48</v>
+      </c>
+      <c r="K49" t="n">
         <v>484</v>
       </c>
-      <c r="L39" t="n">
+      <c r="L49" t="n">
         <v>1</v>
       </c>
-      <c r="M39" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O39" t="inlineStr">
+      <c r="M49" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="1" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="1" t="inlineStr">
         <is>
           <t>EBSD6oME</t>
         </is>
       </c>
-      <c r="B40" s="2" t="n">
+      <c r="B50" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr">
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr">
         <is>
           <t xml:space="preserve">prenton park
   birkenhead </t>
         </is>
       </c>
-      <c r="E40" t="n">
+      <c r="E50" t="n">
         <v>16587</v>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>jVhkb1QE</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="G50" t="inlineStr">
         <is>
           <t>tranmere</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="H50" t="inlineStr">
         <is>
           <t>6ZvdGuYf</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="I50" t="inlineStr">
         <is>
           <t>accrington</t>
         </is>
       </c>
-      <c r="J40" t="n">
-        <v>48</v>
-      </c>
-      <c r="K40" t="n">
+      <c r="J50" t="n">
+        <v>48</v>
+      </c>
+      <c r="K50" t="n">
         <v>484</v>
       </c>
-      <c r="L40" t="n">
+      <c r="L50" t="n">
         <v>1</v>
       </c>
-      <c r="M40" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O40" t="inlineStr">
+      <c r="M50" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="1" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="1" t="inlineStr">
         <is>
           <t>WSQqW4p2</t>
         </is>
       </c>
-      <c r="B41" s="2" t="n">
+      <c r="B51" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr">
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr">
         <is>
           <t xml:space="preserve">bescot stadium
   walsall </t>
         </is>
       </c>
-      <c r="E41" t="n">
+      <c r="E51" t="n">
         <v>11300</v>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F51" t="inlineStr">
         <is>
           <t>YgrfcLuL</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G51" t="inlineStr">
         <is>
           <t>walsall</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H51" t="inlineStr">
         <is>
           <t>ve14a3l4</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I51" t="inlineStr">
         <is>
           <t>exeter</t>
         </is>
       </c>
-      <c r="J41" t="n">
-        <v>48</v>
-      </c>
-      <c r="K41" t="n">
+      <c r="J51" t="n">
+        <v>48</v>
+      </c>
+      <c r="K51" t="n">
         <v>484</v>
       </c>
-      <c r="L41" t="n">
+      <c r="L51" t="n">
         <v>1</v>
       </c>
-      <c r="M41" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O41" t="inlineStr">
+      <c r="M51" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="1" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="1" t="inlineStr">
         <is>
           <t>vaX1LmWq</t>
         </is>
       </c>
-      <c r="B42" s="2" t="n">
+      <c r="B52" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr">
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr">
         <is>
           <t xml:space="preserve">vicarage road
   watford </t>
         </is>
       </c>
-      <c r="E42" t="n">
+      <c r="E52" t="n">
         <v>22200</v>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>UmMRoGzp</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G52" t="inlineStr">
         <is>
           <t>watford</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H52" t="inlineStr">
         <is>
           <t>f9KDxtkU</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="I52" t="inlineStr">
         <is>
           <t>mk dons</t>
         </is>
       </c>
-      <c r="J42" t="n">
-        <v>48</v>
-      </c>
-      <c r="K42" t="n">
+      <c r="J52" t="n">
+        <v>48</v>
+      </c>
+      <c r="K52" t="n">
         <v>484</v>
       </c>
-      <c r="L42" t="n">
+      <c r="L52" t="n">
         <v>1</v>
       </c>
-      <c r="M42" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O42" t="inlineStr">
+      <c r="M52" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="1" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="1" t="inlineStr">
         <is>
           <t>n1hhaOVo</t>
         </is>
       </c>
-      <c r="B43" s="2" t="n">
+      <c r="B53" s="2" t="n">
         <v>45517.65625</v>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr">
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr">
         <is>
           <t xml:space="preserve">dw stadium
   wigan </t>
         </is>
       </c>
-      <c r="E43" t="n">
+      <c r="E53" t="n">
         <v>25133</v>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F53" t="inlineStr">
         <is>
           <t>MgHlK2Na</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="G53" t="inlineStr">
         <is>
           <t>wigan</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="H53" t="inlineStr">
         <is>
           <t>UNGEKMx6</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="I53" t="inlineStr">
         <is>
           <t>barnsley</t>
         </is>
       </c>
-      <c r="J43" t="n">
-        <v>48</v>
-      </c>
-      <c r="K43" t="n">
+      <c r="J53" t="n">
+        <v>48</v>
+      </c>
+      <c r="K53" t="n">
         <v>484</v>
       </c>
-      <c r="L43" t="n">
+      <c r="L53" t="n">
         <v>1</v>
       </c>
-      <c r="M43" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O43" t="inlineStr">
+      <c r="M53" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="1" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
         <is>
           <t>vyoZBtbf</t>
         </is>
       </c>
-      <c r="B44" s="2" t="n">
+      <c r="B54" s="2" t="n">
         <v>45517.66666666666</v>
       </c>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr">
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr">
         <is>
           <t xml:space="preserve">bramall lane
   sheffield </t>
         </is>
       </c>
-      <c r="E44" t="n">
+      <c r="E54" t="n">
         <v>32050</v>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>MeKPSerA</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G54" t="inlineStr">
         <is>
           <t>sheffield utd</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="H54" t="inlineStr">
         <is>
           <t>IgO7K1ZA</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="I54" t="inlineStr">
         <is>
           <t>wrexham</t>
         </is>
       </c>
-      <c r="J44" t="n">
-        <v>48</v>
-      </c>
-      <c r="K44" t="n">
+      <c r="J54" t="n">
+        <v>48</v>
+      </c>
+      <c r="K54" t="n">
         <v>484</v>
       </c>
-      <c r="L44" t="n">
+      <c r="L54" t="n">
         <v>1</v>
       </c>
-      <c r="M44" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O44" t="inlineStr">
+      <c r="M54" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="1" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr">
         <is>
           <t>634r8bcJ</t>
         </is>
       </c>
-      <c r="B45" s="2" t="n">
+      <c r="B55" s="2" t="n">
         <v>45518.65625</v>
       </c>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr">
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr">
         <is>
           <t xml:space="preserve">mkm stadium
   hull </t>
         </is>
       </c>
-      <c r="E45" t="n">
+      <c r="E55" t="n">
         <v>25586</v>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F55" t="inlineStr">
         <is>
           <t>S66R0t75</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G55" t="inlineStr">
         <is>
           <t>hull</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="H55" t="inlineStr">
         <is>
           <t>llcCvIcG</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="I55" t="inlineStr">
         <is>
           <t>sheffield wed</t>
         </is>
       </c>
-      <c r="J45" t="n">
-        <v>48</v>
-      </c>
-      <c r="K45" t="n">
+      <c r="J55" t="n">
+        <v>48</v>
+      </c>
+      <c r="K55" t="n">
         <v>484</v>
       </c>
-      <c r="L45" t="n">
+      <c r="L55" t="n">
         <v>1</v>
       </c>
-      <c r="M45" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O45" t="inlineStr">
+      <c r="M55" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="1" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="1" t="inlineStr">
         <is>
           <t>pbFTwdnB</t>
         </is>
       </c>
-      <c r="B46" s="2" t="n">
+      <c r="B56" s="2" t="n">
         <v>45518.65625</v>
       </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr">
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr">
         <is>
           <t xml:space="preserve">home park
   plymouth </t>
         </is>
       </c>
-      <c r="E46" t="n">
+      <c r="E56" t="n">
         <v>17000</v>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F56" t="inlineStr">
         <is>
           <t>WpGM6ELj</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="G56" t="inlineStr">
         <is>
           <t>plymouth</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="H56" t="inlineStr">
         <is>
           <t>jizXHcsM</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="I56" t="inlineStr">
         <is>
           <t>cheltenham</t>
         </is>
       </c>
-      <c r="J46" t="n">
-        <v>48</v>
-      </c>
-      <c r="K46" t="n">
+      <c r="J56" t="n">
+        <v>48</v>
+      </c>
+      <c r="K56" t="n">
         <v>484</v>
       </c>
-      <c r="L46" t="n">
+      <c r="L56" t="n">
         <v>1</v>
       </c>
-      <c r="M46" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O46" t="inlineStr">
+      <c r="M56" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="1" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="1" t="inlineStr">
         <is>
           <t>697ha3El</t>
         </is>
       </c>
-      <c r="B47" s="2" t="n">
+      <c r="B57" s="2" t="n">
         <v>45518.66666666666</v>
       </c>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr">
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr">
         <is>
           <t xml:space="preserve">elland road
   leeds </t>
         </is>
       </c>
-      <c r="E47" t="n">
+      <c r="E57" t="n">
         <v>37792</v>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F57" t="inlineStr">
         <is>
           <t>tUxUbLR2</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="G57" t="inlineStr">
         <is>
           <t>leeds</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="H57" t="inlineStr">
         <is>
           <t>6F0lvLNC</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="I57" t="inlineStr">
         <is>
           <t>middlesbrough</t>
         </is>
       </c>
-      <c r="J47" t="n">
-        <v>48</v>
-      </c>
-      <c r="K47" t="n">
+      <c r="J57" t="n">
+        <v>48</v>
+      </c>
+      <c r="K57" t="n">
         <v>484</v>
       </c>
-      <c r="L47" t="n">
+      <c r="L57" t="n">
         <v>1</v>
       </c>
-      <c r="M47" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O47" t="inlineStr">
+      <c r="M57" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>

</xml_diff>

<commit_message>
DATA. Ultimo collect_predictions.py antes de salir al mercado.
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
+++ b/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O57"/>
+  <dimension ref="A1:O56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1747,58 +1747,53 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>tYjCfe2E</t>
+          <t>OMDVg8x9</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>45514.45833333334</v>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gillett j 
-  aus </t>
-        </is>
-      </c>
+        <v>45517.64583333334</v>
+      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">wembley stadium
-  london </t>
+          <t xml:space="preserve">brunton park
+  carlisle </t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>90000</v>
+        <v>17949</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Wtn9Stg0</t>
+          <t>dUzTIwSF</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>manchester city</t>
+          <t>carlisle</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>ppjDR086</t>
+          <t>hSUajdSS</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>manchester utd</t>
+          <t>stoke</t>
         </is>
       </c>
       <c r="J22" t="n">
         <v>48</v>
       </c>
       <c r="K22" t="n">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>2024</v>
+        <v>20242025</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
@@ -1807,14 +1802,14 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>fa community shield</t>
+          <t>efl cup</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>OMDVg8x9</t>
+          <t>jXcAnQUr</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
@@ -1823,31 +1818,31 @@
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">brunton park
-  carlisle </t>
+          <t xml:space="preserve">brisbane road
+  london </t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>17949</v>
+        <v>9271</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>dUzTIwSF</t>
+          <t>KKyYcus9</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>carlisle</t>
+          <t>leyton orient</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>hSUajdSS</t>
+          <t>ChwgcrNJ</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>stoke</t>
+          <t>newport</t>
         </is>
       </c>
       <c r="J23" t="n">
@@ -1876,7 +1871,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>jXcAnQUr</t>
+          <t>fRe0c20b</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1885,31 +1880,31 @@
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">brisbane road
-  london </t>
+          <t xml:space="preserve">edgeley park
+  stockport </t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>9271</v>
+        <v>10841</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>KKyYcus9</t>
+          <t>IX6WjNvr</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>leyton orient</t>
+          <t>stockport county</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>ChwgcrNJ</t>
+          <t>6Nl8nagD</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>newport</t>
+          <t>blackburn</t>
         </is>
       </c>
       <c r="J24" t="n">
@@ -1938,40 +1933,40 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>fRe0c20b</t>
+          <t>CnnJp4ae</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>45517.64583333334</v>
+        <v>45517.65625</v>
       </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">edgeley park
-  stockport </t>
+          <t xml:space="preserve">holker street
+  barrow in furness </t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>10841</v>
+        <v>6500</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>IX6WjNvr</t>
+          <t>KKJL7QXd</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>stockport county</t>
+          <t>barrow</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>6Nl8nagD</t>
+          <t>U3lM3y4e</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>blackburn</t>
+          <t>port vale</t>
         </is>
       </c>
       <c r="J25" t="n">
@@ -2000,7 +1995,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>CnnJp4ae</t>
+          <t>bw1zAKS6</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -2009,31 +2004,31 @@
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">holker street
-  barrow in furness </t>
+          <t xml:space="preserve">toughsheet community stadium
+  bolton </t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>6500</v>
+        <v>28723</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>KKJL7QXd</t>
+          <t>Or1bBrWD</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>barrow</t>
+          <t>bolton</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>U3lM3y4e</t>
+          <t>t6G9wMZN</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>port vale</t>
+          <t>mansfield</t>
         </is>
       </c>
       <c r="J26" t="n">
@@ -2062,7 +2057,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>bw1zAKS6</t>
+          <t>GINCsvmn</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
@@ -2071,31 +2066,31 @@
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">toughsheet community stadium
-  bolton </t>
+          <t xml:space="preserve">ashton gate stadium
+  bristol </t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>28723</v>
+        <v>27000</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Or1bBrWD</t>
+          <t>MahqU27I</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>bolton</t>
+          <t>bristol city</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>t6G9wMZN</t>
+          <t>GOvB22xg</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>mansfield</t>
+          <t>coventry</t>
         </is>
       </c>
       <c r="J27" t="n">
@@ -2124,7 +2119,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>GINCsvmn</t>
+          <t>x6klsVh3</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -2133,31 +2128,31 @@
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">ashton gate stadium
-  bristol </t>
+          <t xml:space="preserve">hayes lane
+  london </t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>27000</v>
+        <v>5000</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>MahqU27I</t>
+          <t>Opdcd08Q</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>bristol city</t>
+          <t>bromley</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>GOvB22xg</t>
+          <t>4KREuF43</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>coventry</t>
+          <t>afc wimbledon</t>
         </is>
       </c>
       <c r="J28" t="n">
@@ -2186,7 +2181,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>x6klsVh3</t>
+          <t>b3pRrrU7</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
@@ -2195,31 +2190,31 @@
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">hayes lane
-  london </t>
+          <t xml:space="preserve">pirelli stadium
+  burton upon trent </t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>5000</v>
+        <v>6912</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Opdcd08Q</t>
+          <t>nwCtJaJT</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>bromley</t>
+          <t>burton</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>4KREuF43</t>
+          <t>8EFIJthC</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>afc wimbledon</t>
+          <t>blackpool</t>
         </is>
       </c>
       <c r="J29" t="n">
@@ -2248,7 +2243,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>b3pRrrU7</t>
+          <t>WfkfPdXH</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -2257,31 +2252,31 @@
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">pirelli stadium
-  burton upon trent </t>
+          <t xml:space="preserve">abbey stadium
+  cambridge </t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>6912</v>
+        <v>7937</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>nwCtJaJT</t>
+          <t>lnb8EJRp</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>burton</t>
+          <t>cambridge utd</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>8EFIJthC</t>
+          <t>lrMHUHDc</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>blackpool</t>
+          <t>qpr</t>
         </is>
       </c>
       <c r="J30" t="n">
@@ -2310,7 +2305,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>WfkfPdXH</t>
+          <t>SMr3Nz2U</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
@@ -2319,31 +2314,31 @@
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">abbey stadium
-  cambridge </t>
+          <t xml:space="preserve">cardiff city stadium
+  cardiff </t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>7937</v>
+        <v>33280</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>lnb8EJRp</t>
+          <t>hO8wh6aP</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>cambridge utd</t>
+          <t>cardiff</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>lrMHUHDc</t>
+          <t>GILi6JC9</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>qpr</t>
+          <t>bristol rovers</t>
         </is>
       </c>
       <c r="J31" t="n">
@@ -2372,7 +2367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>SMr3Nz2U</t>
+          <t>xYBLuIHb</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -2381,31 +2376,31 @@
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">cardiff city stadium
-  cardiff </t>
+          <t xml:space="preserve">the valley
+  london </t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>33280</v>
+        <v>27111</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>hO8wh6aP</t>
+          <t>fXf5mQ7t</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>cardiff</t>
+          <t>charlton</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>GILi6JC9</t>
+          <t>SWk4muv7</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>bristol rovers</t>
+          <t>birmingham</t>
         </is>
       </c>
       <c r="J32" t="n">
@@ -2434,7 +2429,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>xYBLuIHb</t>
+          <t>6os5wmhS</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
@@ -2443,31 +2438,31 @@
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">the valley
-  london </t>
+          <t xml:space="preserve">colchester community stadium
+  colchester </t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>27111</v>
+        <v>10105</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>fXf5mQ7t</t>
+          <t>xYu73rNn</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>charlton</t>
+          <t>colchester</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>SWk4muv7</t>
+          <t>EmlVDpVP</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>birmingham</t>
+          <t>reading</t>
         </is>
       </c>
       <c r="J33" t="n">
@@ -2496,7 +2491,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>6os5wmhS</t>
+          <t>Kl7vhn7L</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -2505,31 +2500,31 @@
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">colchester community stadium
-  colchester </t>
+          <t xml:space="preserve">the broadfield stadium
+  crawley </t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>10105</v>
+        <v>6134</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>xYu73rNn</t>
+          <t>QVmLl54o</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>colchester</t>
+          <t>crawley</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>EmlVDpVP</t>
+          <t>xSloasB8</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>reading</t>
+          <t>swindon</t>
         </is>
       </c>
       <c r="J34" t="n">
@@ -2558,7 +2553,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>Kl7vhn7L</t>
+          <t>nw6fJO5K</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
@@ -2567,31 +2562,31 @@
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">the broadfield stadium
-  crawley </t>
+          <t xml:space="preserve">pride park
+  derby </t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>6134</v>
+        <v>33597</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>QVmLl54o</t>
+          <t>Iug0YO0Q</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>crawley</t>
+          <t>derby</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>xSloasB8</t>
+          <t>dQIMIN5n</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>swindon</t>
+          <t>chesterfield</t>
         </is>
       </c>
       <c r="J35" t="n">
@@ -2620,7 +2615,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>nw6fJO5K</t>
+          <t>bHPacsq1</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2629,31 +2624,31 @@
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">pride park
-  derby </t>
+          <t xml:space="preserve">highbury stadium
+  fleetwood </t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>33597</v>
+        <v>5327</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Iug0YO0Q</t>
+          <t>tCZ3D68d</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>derby</t>
+          <t>fleetwood</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>dQIMIN5n</t>
+          <t>CCBWpzjj</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>chesterfield</t>
+          <t>west brom</t>
         </is>
       </c>
       <c r="J36" t="n">
@@ -2682,7 +2677,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>bHPacsq1</t>
+          <t>MwmHgKaN</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
@@ -2691,31 +2686,31 @@
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">highbury stadium
-  fleetwood </t>
+          <t xml:space="preserve">blundell park
+  cleethorpes </t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>5327</v>
+        <v>9052</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>tCZ3D68d</t>
+          <t>OEaiS3za</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>fleetwood</t>
+          <t>grimsby</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>CCBWpzjj</t>
+          <t>bsc3EJ27</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>west brom</t>
+          <t>bradford city</t>
         </is>
       </c>
       <c r="J37" t="n">
@@ -2744,7 +2739,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>MwmHgKaN</t>
+          <t>lQl9etVA</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2753,31 +2748,31 @@
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">blundell park
-  cleethorpes </t>
+          <t xml:space="preserve">john smith s stadium
+  huddersfield </t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>9052</v>
+        <v>24121</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>OEaiS3za</t>
+          <t>xxxpBZl2</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>grimsby</t>
+          <t>huddersfield</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>bsc3EJ27</t>
+          <t>zmKRcPKu</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>bradford city</t>
+          <t>morecambe</t>
         </is>
       </c>
       <c r="J38" t="n">
@@ -2806,7 +2801,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>lQl9etVA</t>
+          <t>KWD8eLDD</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
@@ -2815,31 +2810,31 @@
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">john smith s stadium
-  huddersfield </t>
+          <t xml:space="preserve">lner stadium
+  lincoln </t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>24121</v>
+        <v>10669</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>xxxpBZl2</t>
+          <t>hrHTRs5B</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>huddersfield</t>
+          <t>lincoln</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>zmKRcPKu</t>
+          <t>CQv5qrFt</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>morecambe</t>
+          <t>harrogate</t>
         </is>
       </c>
       <c r="J39" t="n">
@@ -2868,7 +2863,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>KWD8eLDD</t>
+          <t>xUXzYQFk</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2877,31 +2872,31 @@
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">lner stadium
-  lincoln </t>
+          <t xml:space="preserve">sixfields stadium
+  northampton </t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>10669</v>
+        <v>7798</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>hrHTRs5B</t>
+          <t>l4P6dwRR</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>lincoln</t>
+          <t>northampton</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>CQv5qrFt</t>
+          <t>hl2V5JIl</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>harrogate</t>
+          <t>wycombe</t>
         </is>
       </c>
       <c r="J40" t="n">
@@ -2930,7 +2925,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>xUXzYQFk</t>
+          <t>CCV9JR0d</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
@@ -2939,31 +2934,31 @@
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">sixfields stadium
-  northampton </t>
+          <t xml:space="preserve">carrow road
+  norwich </t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>7798</v>
+        <v>27137</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>l4P6dwRR</t>
+          <t>Qo6off6p</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>northampton</t>
+          <t>norwich</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>hl2V5JIl</t>
+          <t>ANwyQM2M</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>wycombe</t>
+          <t>stevenage</t>
         </is>
       </c>
       <c r="J41" t="n">
@@ -2992,7 +2987,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>CCV9JR0d</t>
+          <t>bsinRI25</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -3001,31 +2996,31 @@
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">carrow road
-  norwich </t>
+          <t xml:space="preserve">kassam stadium
+  oxford </t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>27137</v>
+        <v>12500</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Qo6off6p</t>
+          <t>vgOBT43c</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>norwich</t>
+          <t>oxford utd</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>ANwyQM2M</t>
+          <t>tWeI85kh</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>stevenage</t>
+          <t>peterborough</t>
         </is>
       </c>
       <c r="J42" t="n">
@@ -3054,7 +3049,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>bsinRI25</t>
+          <t>GbaVU03t</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
@@ -3063,31 +3058,31 @@
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">kassam stadium
-  oxford </t>
+          <t xml:space="preserve">fratton park
+  portsmouth </t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>12500</v>
+        <v>21944</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>vgOBT43c</t>
+          <t>zckREQFJ</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>oxford utd</t>
+          <t>portsmouth</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>tWeI85kh</t>
+          <t>6uz2cJBL</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>peterborough</t>
+          <t>millwall</t>
         </is>
       </c>
       <c r="J43" t="n">
@@ -3116,7 +3111,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>GbaVU03t</t>
+          <t>tOTmlbNp</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -3125,31 +3120,31 @@
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">fratton park
-  portsmouth </t>
+          <t xml:space="preserve">deepdale
+  preston </t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>21944</v>
+        <v>23408</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>zckREQFJ</t>
+          <t>x8IDVcbi</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>portsmouth</t>
+          <t>preston</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>6uz2cJBL</t>
+          <t>WSzc94ws</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>millwall</t>
+          <t>sunderland</t>
         </is>
       </c>
       <c r="J44" t="n">
@@ -3178,7 +3173,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>tOTmlbNp</t>
+          <t>nPQL4PjR</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
@@ -3187,31 +3182,31 @@
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">deepdale
-  preston </t>
+          <t xml:space="preserve">aesseal new york stadium
+  rotherham </t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>23408</v>
+        <v>12021</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>x8IDVcbi</t>
+          <t>KMfM7P4b</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>preston</t>
+          <t>rotherham</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>WSzc94ws</t>
+          <t>YacqHHdS</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>sunderland</t>
+          <t>crewe</t>
         </is>
       </c>
       <c r="J45" t="n">
@@ -3240,7 +3235,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>nPQL4PjR</t>
+          <t>pWhdu9NF</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -3249,31 +3244,31 @@
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">aesseal new york stadium
-  rotherham </t>
+          <t xml:space="preserve">peninsula stadium
+  salford </t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>12021</v>
+        <v>5108</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>KMfM7P4b</t>
+          <t>W4AadhN3</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>rotherham</t>
+          <t>salford</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>YacqHHdS</t>
+          <t>hlzYDy5q</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>crewe</t>
+          <t>doncaster</t>
         </is>
       </c>
       <c r="J46" t="n">
@@ -3302,7 +3297,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>pWhdu9NF</t>
+          <t>6NnRD2Ts</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
@@ -3311,31 +3306,31 @@
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">peninsula stadium
-  salford </t>
+          <t xml:space="preserve">the croud meadow
+  shrewsbury </t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>5108</v>
+        <v>9877</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>W4AadhN3</t>
+          <t>EqfQ6qK4</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>salford</t>
+          <t>shrewsbury</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>hlzYDy5q</t>
+          <t>EwJVdqzn</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>doncaster</t>
+          <t>notts co</t>
         </is>
       </c>
       <c r="J47" t="n">
@@ -3364,7 +3359,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>6NnRD2Ts</t>
+          <t>2FcwTvYh</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -3373,31 +3368,31 @@
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">the croud meadow
-  shrewsbury </t>
+          <t xml:space="preserve">swansea com stadium
+  swansea </t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>9877</v>
+        <v>21088</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>EqfQ6qK4</t>
+          <t>K6xezbY7</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>shrewsbury</t>
+          <t>swansea</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>EwJVdqzn</t>
+          <t>WvZyDeKk</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>notts co</t>
+          <t>gillingham</t>
         </is>
       </c>
       <c r="J48" t="n">
@@ -3426,7 +3421,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>2FcwTvYh</t>
+          <t>EBSD6oME</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
@@ -3435,31 +3430,31 @@
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">swansea com stadium
-  swansea </t>
+          <t xml:space="preserve">prenton park
+  birkenhead </t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>21088</v>
+        <v>16587</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>K6xezbY7</t>
+          <t>jVhkb1QE</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>swansea</t>
+          <t>tranmere</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>WvZyDeKk</t>
+          <t>6ZvdGuYf</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>gillingham</t>
+          <t>accrington</t>
         </is>
       </c>
       <c r="J49" t="n">
@@ -3488,7 +3483,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>EBSD6oME</t>
+          <t>WSQqW4p2</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -3497,31 +3492,31 @@
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">prenton park
-  birkenhead </t>
+          <t xml:space="preserve">bescot stadium
+  walsall </t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>16587</v>
+        <v>11300</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>jVhkb1QE</t>
+          <t>YgrfcLuL</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>tranmere</t>
+          <t>walsall</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>6ZvdGuYf</t>
+          <t>ve14a3l4</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>accrington</t>
+          <t>exeter</t>
         </is>
       </c>
       <c r="J50" t="n">
@@ -3550,7 +3545,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>WSQqW4p2</t>
+          <t>vaX1LmWq</t>
         </is>
       </c>
       <c r="B51" s="2" t="n">
@@ -3559,31 +3554,31 @@
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">bescot stadium
-  walsall </t>
+          <t xml:space="preserve">vicarage road
+  watford </t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>11300</v>
+        <v>22200</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>YgrfcLuL</t>
+          <t>UmMRoGzp</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>walsall</t>
+          <t>watford</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>ve14a3l4</t>
+          <t>f9KDxtkU</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>exeter</t>
+          <t>mk dons</t>
         </is>
       </c>
       <c r="J51" t="n">
@@ -3612,7 +3607,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>vaX1LmWq</t>
+          <t>n1hhaOVo</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -3621,31 +3616,31 @@
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">vicarage road
-  watford </t>
+          <t xml:space="preserve">the brick community stadium
+  wigan </t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>22200</v>
+        <v>25133</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>UmMRoGzp</t>
+          <t>MgHlK2Na</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>watford</t>
+          <t>wigan</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>f9KDxtkU</t>
+          <t>UNGEKMx6</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>mk dons</t>
+          <t>barnsley</t>
         </is>
       </c>
       <c r="J52" t="n">
@@ -3674,40 +3669,40 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>n1hhaOVo</t>
+          <t>vyoZBtbf</t>
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>45517.65625</v>
+        <v>45517.66666666666</v>
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">dw stadium
-  wigan </t>
+          <t xml:space="preserve">bramall lane
+  sheffield </t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>25133</v>
+        <v>32050</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>MgHlK2Na</t>
+          <t>MeKPSerA</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>wigan</t>
+          <t>sheffield utd</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>UNGEKMx6</t>
+          <t>IgO7K1ZA</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>barnsley</t>
+          <t>wrexham</t>
         </is>
       </c>
       <c r="J53" t="n">
@@ -3736,40 +3731,40 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>vyoZBtbf</t>
+          <t>634r8bcJ</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>45517.66666666666</v>
+        <v>45518.65625</v>
       </c>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
-          <t xml:space="preserve">bramall lane
-  sheffield </t>
+          <t xml:space="preserve">mkm stadium
+  hull </t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>32050</v>
+        <v>25586</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>MeKPSerA</t>
+          <t>S66R0t75</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>sheffield utd</t>
+          <t>hull</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>IgO7K1ZA</t>
+          <t>llcCvIcG</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>wrexham</t>
+          <t>sheffield wed</t>
         </is>
       </c>
       <c r="J54" t="n">
@@ -3798,7 +3793,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>634r8bcJ</t>
+          <t>pbFTwdnB</t>
         </is>
       </c>
       <c r="B55" s="2" t="n">
@@ -3807,31 +3802,31 @@
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">mkm stadium
-  hull </t>
+          <t xml:space="preserve">home park
+  plymouth </t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>25586</v>
+        <v>17000</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>S66R0t75</t>
+          <t>WpGM6ELj</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>hull</t>
+          <t>plymouth</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>llcCvIcG</t>
+          <t>jizXHcsM</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>sheffield wed</t>
+          <t>cheltenham</t>
         </is>
       </c>
       <c r="J55" t="n">
@@ -3860,40 +3855,40 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>pbFTwdnB</t>
+          <t>697ha3El</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>45518.65625</v>
+        <v>45518.66666666666</v>
       </c>
       <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">home park
-  plymouth </t>
+          <t xml:space="preserve">elland road
+  leeds </t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>17000</v>
+        <v>37792</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>WpGM6ELj</t>
+          <t>tUxUbLR2</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>plymouth</t>
+          <t>leeds</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>jizXHcsM</t>
+          <t>6F0lvLNC</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>cheltenham</t>
+          <t>middlesbrough</t>
         </is>
       </c>
       <c r="J56" t="n">
@@ -3914,68 +3909,6 @@
         </is>
       </c>
       <c r="O56" t="inlineStr">
-        <is>
-          <t>efl cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="1" t="inlineStr">
-        <is>
-          <t>697ha3El</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="n">
-        <v>45518.66666666666</v>
-      </c>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">elland road
-  leeds </t>
-        </is>
-      </c>
-      <c r="E57" t="n">
-        <v>37792</v>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>tUxUbLR2</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>leeds</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>6F0lvLNC</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>middlesbrough</t>
-        </is>
-      </c>
-      <c r="J57" t="n">
-        <v>48</v>
-      </c>
-      <c r="K57" t="n">
-        <v>484</v>
-      </c>
-      <c r="L57" t="n">
-        <v>1</v>
-      </c>
-      <c r="M57" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N57" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O57" t="inlineStr">
         <is>
           <t>efl cup</t>
         </is>

</xml_diff>

<commit_message>
Nuevo assess tras evitar dp + Seleccion nuevos modelos
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
+++ b/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,45 +507,45 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>8j9FTL56</t>
+          <t>6RCbX36s</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45528.35416666666</v>
+        <v>45529.41666666666</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">pawson c 
+          <t xml:space="preserve">coote d 
   eng </t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">amex stadium
-  brighton </t>
+          <t xml:space="preserve">vitality stadium
+  bournemouth </t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>31876</v>
+        <v>11307</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2XrRecc3</t>
+          <t>OtpNdwrc</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>brighton</t>
+          <t>bournemouth</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>ppjDR086</t>
+          <t>p6ahwuwJ</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>manchester utd</t>
+          <t>newcastle</t>
         </is>
       </c>
       <c r="J2" t="n">
@@ -574,45 +574,45 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>U5cORazJ</t>
+          <t>61T7bt5t</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45528.45833333334</v>
+        <v>45529.41666666666</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">jones r 
+          <t xml:space="preserve">england d 
   eng </t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">selhurst park
-  london </t>
+          <t xml:space="preserve">molineux stadium
+  wolverhampton </t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>25486</v>
+        <v>31750</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>AovF1Mia</t>
+          <t>j3Azpf5d</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>crystal palace</t>
+          <t>wolves</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Cxq57r8g</t>
+          <t>4fGZN2oK</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>west ham</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="J3" t="n">
@@ -641,45 +641,45 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>dCkAk3SP</t>
+          <t>GdWtpsjm</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45528.45833333334</v>
+        <v>45529.52083333334</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">bond d 
+          <t xml:space="preserve">attwell s 
   eng </t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">craven cottage
-  london </t>
+          <t xml:space="preserve">anfield
+  liverpool </t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>26600</v>
+        <v>61276</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>69ZiU2Om</t>
+          <t>lId4TMwf</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>fulham</t>
+          <t>liverpool</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>KrrdAMyI</t>
+          <t>xYe7DwID</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>leicester</t>
+          <t>brentford</t>
         </is>
       </c>
       <c r="J4" t="n">
@@ -708,45 +708,40 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>lAUlrLKa</t>
+          <t>ERWFdKZh</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45528.45833333334</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">salisbury m 
-  eng </t>
-        </is>
-      </c>
+        <v>45535.35416666666</v>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">etihad stadium
-  manchester </t>
+          <t xml:space="preserve">emirates stadium
+  london </t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>55097</v>
+        <v>60704</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Wtn9Stg0</t>
+          <t>hA1Zm19f</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>manchester city</t>
+          <t>arsenal</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>thqhB2MB</t>
+          <t>2XrRecc3</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>ipswich</t>
+          <t>brighton</t>
         </is>
       </c>
       <c r="J5" t="n">
@@ -775,45 +770,40 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>fNaktakC</t>
+          <t>8QPOfb45</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45528.45833333334</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">barrott s 
-  eng </t>
-        </is>
-      </c>
+        <v>45535.45833333334</v>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">st  mary s stadium
-  southampton </t>
+          <t xml:space="preserve">brentford community stadium
+  london </t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>32384</v>
+        <v>17250</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
+          <t>xYe7DwID</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>brentford</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>WdKOwxDM</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>southampton</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>UsushcZr</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>nottingham</t>
         </is>
       </c>
       <c r="J6" t="n">
@@ -842,45 +832,40 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>2m3cvwKO</t>
+          <t>x6HuiG3U</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>45528.45833333334</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">taylor a 
-  eng </t>
-        </is>
-      </c>
+        <v>45535.45833333334</v>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">tottenham hotspur stadium
-  london </t>
+          <t xml:space="preserve">goodison park
+  liverpool </t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>62850</v>
+        <v>39572</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>UDg08Ohm</t>
+          <t>KluSTr9s</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>tottenham</t>
+          <t>everton</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>KluSTr9s</t>
+          <t>OtpNdwrc</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>everton</t>
+          <t>bournemouth</t>
         </is>
       </c>
       <c r="J7" t="n">
@@ -909,45 +894,40 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>2g67Vsyf</t>
+          <t>SUdkBJln</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>45528.5625</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">oliver m 
-  eng </t>
-        </is>
-      </c>
+        <v>45535.45833333334</v>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">villa park
-  birmingham </t>
+          <t xml:space="preserve">portman road
+  ipswich </t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>42789</v>
+        <v>29673</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>W00wmLO0</t>
+          <t>thqhB2MB</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>aston villa</t>
+          <t>ipswich</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>hA1Zm19f</t>
+          <t>69ZiU2Om</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>arsenal</t>
+          <t>fulham</t>
         </is>
       </c>
       <c r="J8" t="n">
@@ -968,6 +948,378 @@
         </is>
       </c>
       <c r="O8" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>lpob9cJb</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>45535.45833333334</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king power stadium
+  leicester </t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>32261</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>KrrdAMyI</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>leicester</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>W00wmLO0</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>aston villa</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>48</v>
+      </c>
+      <c r="K9" t="n">
+        <v>481</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>2Fanm72d</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>45535.45833333334</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">city ground
+  nottingham </t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>30404</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>UsushcZr</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>nottingham</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>j3Azpf5d</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>wolves</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>48</v>
+      </c>
+      <c r="K10" t="n">
+        <v>481</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>INsZAAf3</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>45535.5625</v>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">london stadium
+  london </t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>62500</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Cxq57r8g</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>west ham</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Wtn9Stg0</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>manchester city</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>48</v>
+      </c>
+      <c r="K11" t="n">
+        <v>481</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>tvOWhxZH</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>45536.39583333334</v>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stamford bridge
+  london </t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>40341</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>4fGZN2oK</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>chelsea</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>AovF1Mia</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>crystal palace</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>48</v>
+      </c>
+      <c r="K12" t="n">
+        <v>481</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>U11vkTXq</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>45536.39583333334</v>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">st  james  park
+  newcastle </t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>52305</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>p6ahwuwJ</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>newcastle</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>UDg08Ohm</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>tottenham</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>48</v>
+      </c>
+      <c r="K13" t="n">
+        <v>481</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>z1q67ylB</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>45536.5</v>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">old trafford
+  manchester </t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>75635</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>ppjDR086</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>manchester utd</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>lId4TMwf</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>liverpool</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>48</v>
+      </c>
+      <c r="K14" t="n">
+        <v>481</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
         <is>
           <t>premier league</t>
         </is>

</xml_diff>

<commit_message>
DATA. Nuevo assess models tras partidos del fin de semana
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
+++ b/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,45 +507,40 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>tvOWhxZH</t>
+          <t>2kGeEq1e</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45536.39583333334</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gillett j 
-  aus </t>
-        </is>
-      </c>
+        <v>45549.35416666666</v>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">stamford bridge
-  london </t>
+          <t xml:space="preserve">st  mary s stadium
+  southampton </t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>40341</v>
+        <v>32384</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>4fGZN2oK</t>
+          <t>WdKOwxDM</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>chelsea</t>
+          <t>southampton</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>AovF1Mia</t>
+          <t>ppjDR086</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>crystal palace</t>
+          <t>manchester utd</t>
         </is>
       </c>
       <c r="J2" t="n">
@@ -574,45 +569,40 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>U11vkTXq</t>
+          <t>2TvL16Hk</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45536.39583333334</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">jones r 
-  eng </t>
-        </is>
-      </c>
+        <v>45549.45833333334</v>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">st  james  park
-  newcastle </t>
+          <t xml:space="preserve">amex stadium
+  brighton </t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>52305</v>
+        <v>31876</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>p6ahwuwJ</t>
+          <t>2XrRecc3</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>newcastle</t>
+          <t>brighton</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>UDg08Ohm</t>
+          <t>thqhB2MB</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>tottenham</t>
+          <t>ipswich</t>
         </is>
       </c>
       <c r="J3" t="n">
@@ -641,45 +631,40 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>z1q67ylB</t>
+          <t>beYTapn2</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45536.5</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">taylor a 
-  eng </t>
-        </is>
-      </c>
+        <v>45549.45833333334</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">old trafford
-  manchester </t>
+          <t xml:space="preserve">selhurst park
+  london </t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>75635</v>
+        <v>25486</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>ppjDR086</t>
+          <t>AovF1Mia</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>manchester utd</t>
+          <t>crystal palace</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>lId4TMwf</t>
+          <t>KrrdAMyI</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>leicester</t>
         </is>
       </c>
       <c r="J4" t="n">
@@ -700,6 +685,440 @@
         </is>
       </c>
       <c r="O4" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>jkLFNmv9</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>45549.45833333334</v>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">craven cottage
+  london </t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>26600</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>69ZiU2Om</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>fulham</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Cxq57r8g</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>west ham</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>48</v>
+      </c>
+      <c r="K5" t="n">
+        <v>481</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>AiyHLR8L</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>45549.45833333334</v>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">anfield
+  liverpool </t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>61276</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>lId4TMwf</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>liverpool</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>UsushcZr</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>nottingham</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>48</v>
+      </c>
+      <c r="K6" t="n">
+        <v>481</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>tzSnG5Wr</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>45549.45833333334</v>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">etihad stadium
+  manchester </t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>55097</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Wtn9Stg0</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>manchester city</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>xYe7DwID</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>brentford</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>48</v>
+      </c>
+      <c r="K7" t="n">
+        <v>481</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Wplk7SgS</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>45549.5625</v>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">villa park
+  birmingham </t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>42789</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>W00wmLO0</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>aston villa</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>KluSTr9s</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>everton</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>48</v>
+      </c>
+      <c r="K8" t="n">
+        <v>481</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>AVat9lPF</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>45549.66666666666</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vitality stadium
+  bournemouth </t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>11307</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>OtpNdwrc</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>bournemouth</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>4fGZN2oK</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>chelsea</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>48</v>
+      </c>
+      <c r="K9" t="n">
+        <v>481</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>AFJ3CNV7</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>45550.41666666666</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tottenham hotspur stadium
+  london </t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>62850</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>UDg08Ohm</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>tottenham</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>hA1Zm19f</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>arsenal</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>48</v>
+      </c>
+      <c r="K10" t="n">
+        <v>481</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>Of1jzRNE</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>45550.52083333334</v>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">molineux stadium
+  wolverhampton </t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>31750</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>j3Azpf5d</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>wolves</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>p6ahwuwJ</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>newcastle</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>48</v>
+      </c>
+      <c r="K11" t="n">
+        <v>481</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
         <is>
           <t>premier league</t>
         </is>

</xml_diff>

<commit_message>
DATA. Selección de modelos tras nuevo assess y nuevos modelos en FRA, ENG, GER y USA.
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
+++ b/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1124,6 +1124,626 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>C0axT3Xo</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>45556.35416666666</v>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">london stadium
+  london </t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>62500</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Cxq57r8g</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>west ham</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>4fGZN2oK</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>chelsea</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>48</v>
+      </c>
+      <c r="K12" t="n">
+        <v>481</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>d8abY4hR</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>45556.45833333334</v>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">villa park
+  birmingham </t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>42789</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>W00wmLO0</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>aston villa</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>j3Azpf5d</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>wolves</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>48</v>
+      </c>
+      <c r="K13" t="n">
+        <v>481</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>pYXoP0FD</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>45556.45833333334</v>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">craven cottage
+  london </t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>26600</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>69ZiU2Om</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>fulham</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>p6ahwuwJ</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>newcastle</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>48</v>
+      </c>
+      <c r="K14" t="n">
+        <v>481</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>xtzXn47K</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>45556.45833333334</v>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king power stadium
+  leicester </t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>32261</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>KrrdAMyI</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>leicester</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>KluSTr9s</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>everton</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>48</v>
+      </c>
+      <c r="K15" t="n">
+        <v>481</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>dQG3srVs</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>45556.45833333334</v>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">anfield
+  liverpool </t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>61276</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>lId4TMwf</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>liverpool</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>OtpNdwrc</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>bournemouth</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>48</v>
+      </c>
+      <c r="K16" t="n">
+        <v>481</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>Q58Kw0U6</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>45556.45833333334</v>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">st  mary s stadium
+  southampton </t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>32384</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>WdKOwxDM</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>southampton</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>thqhB2MB</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>ipswich</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>48</v>
+      </c>
+      <c r="K17" t="n">
+        <v>481</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>W2BSyvaJ</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>45556.45833333334</v>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tottenham hotspur stadium
+  london </t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>62850</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>UDg08Ohm</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>tottenham</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>xYe7DwID</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>brentford</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>48</v>
+      </c>
+      <c r="K18" t="n">
+        <v>481</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>OIqwRMp1</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>45556.5625</v>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">selhurst park
+  london </t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>25486</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>AovF1Mia</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>crystal palace</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>ppjDR086</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>manchester utd</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>48</v>
+      </c>
+      <c r="K19" t="n">
+        <v>481</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>GhtVSrGl</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>45557.41666666666</v>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">amex stadium
+  brighton </t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>31876</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2XrRecc3</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>brighton</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>UsushcZr</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>nottingham</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>48</v>
+      </c>
+      <c r="K20" t="n">
+        <v>481</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>UwFBuMaf</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>45557.52083333334</v>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">etihad stadium
+  manchester </t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>55097</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Wtn9Stg0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>manchester city</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>hA1Zm19f</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>arsenal</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>48</v>
+      </c>
+      <c r="K21" t="n">
+        <v>481</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
DATA. Entrenamiento modelos con nueva preparacion
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
+++ b/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,45 +507,40 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>AFJ3CNV7</t>
+          <t>8MkyzwoT</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45550.41666666666</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gillett j 
-  aus </t>
-        </is>
-      </c>
+        <v>45563.35416666666</v>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">tottenham hotspur stadium
-  london </t>
+          <t xml:space="preserve">st  james  park
+  newcastle </t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>62850</v>
+        <v>52305</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>UDg08Ohm</t>
+          <t>p6ahwuwJ</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>tottenham</t>
+          <t>newcastle</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>hA1Zm19f</t>
+          <t>Wtn9Stg0</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>arsenal</t>
+          <t>manchester city</t>
         </is>
       </c>
       <c r="J2" t="n">
@@ -574,65 +569,1176 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Of1jzRNE</t>
+          <t>GhdgPLWA</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45550.52083333334</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">kavanagh c 
-  eng </t>
-        </is>
-      </c>
+        <v>45563.45833333334</v>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">emirates stadium
+  london </t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>60704</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>hA1Zm19f</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>arsenal</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>KrrdAMyI</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>leicester</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>48</v>
+      </c>
+      <c r="K3" t="n">
+        <v>481</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>l6f1Na1N</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>45563.45833333334</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">brentford community stadium
+  london </t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>17250</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>xYe7DwID</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>brentford</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Cxq57r8g</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>west ham</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>48</v>
+      </c>
+      <c r="K4" t="n">
+        <v>481</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>WQcQHwPp</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>45563.45833333334</v>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stamford bridge
+  london </t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>40341</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>4fGZN2oK</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>chelsea</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2XrRecc3</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>brighton</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>48</v>
+      </c>
+      <c r="K5" t="n">
+        <v>481</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>bXkCusHi</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>45563.45833333334</v>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">goodison park
+  liverpool </t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>39572</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>KluSTr9s</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>everton</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>AovF1Mia</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>crystal palace</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>48</v>
+      </c>
+      <c r="K6" t="n">
+        <v>481</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>4hy7UG8j</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>45563.45833333334</v>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">city ground
+  nottingham </t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>30404</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>UsushcZr</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>nottingham</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>69ZiU2Om</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>fulham</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>48</v>
+      </c>
+      <c r="K7" t="n">
+        <v>481</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>K0JghK0c</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>45563.5625</v>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
         <is>
           <t xml:space="preserve">molineux stadium
   wolverhampton </t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E8" t="n">
         <v>31750</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>j3Azpf5d</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>wolves</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>lId4TMwf</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>liverpool</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>48</v>
+      </c>
+      <c r="K8" t="n">
+        <v>481</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>KnvLwLo4</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>45564.41666666666</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">portman road
+  ipswich </t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>29673</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>thqhB2MB</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>ipswich</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>W00wmLO0</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>aston villa</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>48</v>
+      </c>
+      <c r="K9" t="n">
+        <v>481</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>SCsTyaGG</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>45564.52083333334</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">old trafford
+  manchester </t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>75635</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ppjDR086</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>manchester utd</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>UDg08Ohm</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>tottenham</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>48</v>
+      </c>
+      <c r="K10" t="n">
+        <v>481</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>KQ2pRs2b</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>45565.66666666666</v>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vitality stadium
+  bournemouth </t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>11307</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>OtpNdwrc</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>bournemouth</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>WdKOwxDM</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>southampton</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>48</v>
+      </c>
+      <c r="K11" t="n">
+        <v>481</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>r3Wq3yFF</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>45570.35416666666</v>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">selhurst park
+  london </t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>25486</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>AovF1Mia</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>crystal palace</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>lId4TMwf</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>liverpool</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>48</v>
+      </c>
+      <c r="K12" t="n">
+        <v>481</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>SQM1jbV9</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>45570.45833333334</v>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">emirates stadium
+  london </t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>60704</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>hA1Zm19f</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>arsenal</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>WdKOwxDM</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>southampton</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>48</v>
+      </c>
+      <c r="K13" t="n">
+        <v>481</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>bFdtqGNq</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>45570.45833333334</v>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">brentford community stadium
+  london </t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>17250</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>xYe7DwID</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>brentford</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>j3Azpf5d</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>wolves</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>48</v>
+      </c>
+      <c r="K14" t="n">
+        <v>481</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>YXAOeg7k</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>45570.45833333334</v>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king power stadium
+  leicester </t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>32261</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>KrrdAMyI</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>leicester</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>OtpNdwrc</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>bournemouth</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>48</v>
+      </c>
+      <c r="K15" t="n">
+        <v>481</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>tbEWgXy2</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>45570.45833333334</v>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">etihad stadium
+  manchester </t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>55097</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Wtn9Stg0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>manchester city</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>69ZiU2Om</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>fulham</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>48</v>
+      </c>
+      <c r="K16" t="n">
+        <v>481</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>d6dJHzU8</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>45570.45833333334</v>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">london stadium
+  london </t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>62500</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Cxq57r8g</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>west ham</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>thqhB2MB</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>ipswich</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>48</v>
+      </c>
+      <c r="K17" t="n">
+        <v>481</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>l0Zi1FqS</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>45570.5625</v>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">goodison park
+  liverpool </t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>39572</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>KluSTr9s</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>everton</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>p6ahwuwJ</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>newcastle</t>
         </is>
       </c>
-      <c r="J3" t="n">
-        <v>48</v>
-      </c>
-      <c r="K3" t="n">
-        <v>481</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
+      <c r="J18" t="n">
+        <v>48</v>
+      </c>
+      <c r="K18" t="n">
+        <v>481</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>ltBAlx0M</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>45571.41666666666</v>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">villa park
+  birmingham </t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>42789</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>W00wmLO0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>aston villa</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>ppjDR086</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>manchester utd</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>48</v>
+      </c>
+      <c r="K19" t="n">
+        <v>481</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>nywy5cp3</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>45571.41666666666</v>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stamford bridge
+  london </t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>40341</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>4fGZN2oK</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>chelsea</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>UsushcZr</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>nottingham</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>48</v>
+      </c>
+      <c r="K20" t="n">
+        <v>481</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>fsjksfhd</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>45571.52083333334</v>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">amex stadium
+  brighton </t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>31876</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2XrRecc3</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>brighton</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>UDg08Ohm</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>tottenham</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>48</v>
+      </c>
+      <c r="K21" t="n">
+        <v>481</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
         <is>
           <t>premier league</t>
         </is>

</xml_diff>

<commit_message>
Actualizo predicciones.xlsx por partidos missing en SPA, info de jugadores missing y por cambio en cuotas.
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
+++ b/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,7 +513,12 @@
       <c r="B2" s="2" t="n">
         <v>45563.35416666666</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gillett j 
+  aus </t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t xml:space="preserve">st  james  park
@@ -575,7 +580,12 @@
       <c r="B3" s="2" t="n">
         <v>45563.45833333334</v>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">barrott s 
+  eng </t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t xml:space="preserve">emirates stadium
@@ -637,7 +647,12 @@
       <c r="B4" s="2" t="n">
         <v>45563.45833333334</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hooper s 
+  eng </t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
           <t xml:space="preserve">brentford community stadium
@@ -699,7 +714,12 @@
       <c r="B5" s="2" t="n">
         <v>45563.45833333334</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bankes p 
+  eng </t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
           <t xml:space="preserve">stamford bridge
@@ -761,7 +781,12 @@
       <c r="B6" s="2" t="n">
         <v>45563.45833333334</v>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">madley a 
+  eng </t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
           <t xml:space="preserve">goodison park
@@ -823,7 +848,12 @@
       <c r="B7" s="2" t="n">
         <v>45563.45833333334</v>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">smith j 
+  eng </t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
           <t xml:space="preserve">city ground
@@ -885,7 +915,12 @@
       <c r="B8" s="2" t="n">
         <v>45563.5625</v>
       </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">taylor a 
+  eng </t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
           <t xml:space="preserve">molineux stadium
@@ -947,7 +982,12 @@
       <c r="B9" s="2" t="n">
         <v>45564.41666666666</v>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">attwell s 
+  eng </t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
           <t xml:space="preserve">portman road
@@ -1009,7 +1049,12 @@
       <c r="B10" s="2" t="n">
         <v>45564.52083333334</v>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kavanagh c 
+  eng </t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
           <t xml:space="preserve">old trafford
@@ -1057,688 +1102,6 @@
         </is>
       </c>
       <c r="O10" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>KQ2pRs2b</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>45565.66666666666</v>
-      </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">vitality stadium
-  bournemouth </t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>11307</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>OtpNdwrc</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>bournemouth</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>WdKOwxDM</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>southampton</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
-        <v>48</v>
-      </c>
-      <c r="K11" t="n">
-        <v>481</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>r3Wq3yFF</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>45570.35416666666</v>
-      </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">selhurst park
-  london </t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>25486</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>AovF1Mia</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>crystal palace</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>lId4TMwf</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>liverpool</t>
-        </is>
-      </c>
-      <c r="J12" t="n">
-        <v>48</v>
-      </c>
-      <c r="K12" t="n">
-        <v>481</v>
-      </c>
-      <c r="L12" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>SQM1jbV9</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>45570.45833333334</v>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">emirates stadium
-  london </t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>60704</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>hA1Zm19f</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>arsenal</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>WdKOwxDM</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>southampton</t>
-        </is>
-      </c>
-      <c r="J13" t="n">
-        <v>48</v>
-      </c>
-      <c r="K13" t="n">
-        <v>481</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>bFdtqGNq</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>45570.45833333334</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">brentford community stadium
-  london </t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>17250</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>xYe7DwID</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>brentford</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>j3Azpf5d</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>wolves</t>
-        </is>
-      </c>
-      <c r="J14" t="n">
-        <v>48</v>
-      </c>
-      <c r="K14" t="n">
-        <v>481</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>YXAOeg7k</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>45570.45833333334</v>
-      </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">king power stadium
-  leicester </t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>32261</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>KrrdAMyI</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>leicester</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>OtpNdwrc</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>bournemouth</t>
-        </is>
-      </c>
-      <c r="J15" t="n">
-        <v>48</v>
-      </c>
-      <c r="K15" t="n">
-        <v>481</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>tbEWgXy2</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>45570.45833333334</v>
-      </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">etihad stadium
-  manchester </t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>55097</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Wtn9Stg0</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>manchester city</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>69ZiU2Om</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>fulham</t>
-        </is>
-      </c>
-      <c r="J16" t="n">
-        <v>48</v>
-      </c>
-      <c r="K16" t="n">
-        <v>481</v>
-      </c>
-      <c r="L16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>d6dJHzU8</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>45570.45833333334</v>
-      </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">london stadium
-  london </t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>62500</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Cxq57r8g</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>west ham</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>thqhB2MB</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>ipswich</t>
-        </is>
-      </c>
-      <c r="J17" t="n">
-        <v>48</v>
-      </c>
-      <c r="K17" t="n">
-        <v>481</v>
-      </c>
-      <c r="L17" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>l0Zi1FqS</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>45570.5625</v>
-      </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">goodison park
-  liverpool </t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>39572</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>KluSTr9s</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>everton</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>p6ahwuwJ</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>newcastle</t>
-        </is>
-      </c>
-      <c r="J18" t="n">
-        <v>48</v>
-      </c>
-      <c r="K18" t="n">
-        <v>481</v>
-      </c>
-      <c r="L18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>ltBAlx0M</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="n">
-        <v>45571.41666666666</v>
-      </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">villa park
-  birmingham </t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>42789</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>W00wmLO0</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>aston villa</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>ppjDR086</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>manchester utd</t>
-        </is>
-      </c>
-      <c r="J19" t="n">
-        <v>48</v>
-      </c>
-      <c r="K19" t="n">
-        <v>481</v>
-      </c>
-      <c r="L19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>nywy5cp3</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="n">
-        <v>45571.41666666666</v>
-      </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">stamford bridge
-  london </t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>40341</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>4fGZN2oK</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>chelsea</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>UsushcZr</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>nottingham</t>
-        </is>
-      </c>
-      <c r="J20" t="n">
-        <v>48</v>
-      </c>
-      <c r="K20" t="n">
-        <v>481</v>
-      </c>
-      <c r="L20" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>fsjksfhd</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>45571.52083333334</v>
-      </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">amex stadium
-  brighton </t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>31876</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>2XrRecc3</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>brighton</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>UDg08Ohm</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>tottenham</t>
-        </is>
-      </c>
-      <c r="J21" t="n">
-        <v>48</v>
-      </c>
-      <c r="K21" t="n">
-        <v>481</v>
-      </c>
-      <c r="L21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
         <is>
           <t>premier league</t>
         </is>

</xml_diff>

<commit_message>
Actualizo predicciones.xlsx al cambiar m_to_use
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
+++ b/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,45 +507,45 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>8MkyzwoT</t>
+          <t>KnvLwLo4</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45563.35416666666</v>
+        <v>45564.41666666666</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">gillett j 
-  aus </t>
+          <t xml:space="preserve">attwell s 
+  eng </t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">st  james  park
-  newcastle </t>
+          <t xml:space="preserve">portman road
+  ipswich </t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>52305</v>
+        <v>29673</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>p6ahwuwJ</t>
+          <t>thqhB2MB</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>newcastle</t>
+          <t>ipswich</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Wtn9Stg0</t>
+          <t>W00wmLO0</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>manchester city</t>
+          <t>aston villa</t>
         </is>
       </c>
       <c r="J2" t="n">
@@ -574,45 +574,45 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>GhdgPLWA</t>
+          <t>SCsTyaGG</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45563.45833333334</v>
+        <v>45564.52083333334</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">barrott s 
+          <t xml:space="preserve">kavanagh c 
   eng </t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">emirates stadium
-  london </t>
+          <t xml:space="preserve">old trafford
+  manchester </t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>60704</v>
+        <v>75635</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>hA1Zm19f</t>
+          <t>ppjDR086</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>arsenal</t>
+          <t>manchester utd</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>KrrdAMyI</t>
+          <t>UDg08Ohm</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>leicester</t>
+          <t>tottenham</t>
         </is>
       </c>
       <c r="J3" t="n">
@@ -641,45 +641,45 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>l6f1Na1N</t>
+          <t>KQ2pRs2b</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45563.45833333334</v>
+        <v>45565.66666666666</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">hooper s 
+          <t xml:space="preserve">oliver m 
   eng </t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">brentford community stadium
-  london </t>
+          <t xml:space="preserve">vitality stadium
+  bournemouth </t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>17250</v>
+        <v>11307</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>xYe7DwID</t>
+          <t>OtpNdwrc</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>brentford</t>
+          <t>bournemouth</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Cxq57r8g</t>
+          <t>WdKOwxDM</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>west ham</t>
+          <t>southampton</t>
         </is>
       </c>
       <c r="J4" t="n">
@@ -700,408 +700,6 @@
         </is>
       </c>
       <c r="O4" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>WQcQHwPp</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>45563.45833333334</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bankes p 
-  eng </t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">stamford bridge
-  london </t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>40341</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>4fGZN2oK</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>chelsea</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2XrRecc3</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>brighton</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>48</v>
-      </c>
-      <c r="K5" t="n">
-        <v>481</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>bXkCusHi</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>45563.45833333334</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">madley a 
-  eng </t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">goodison park
-  liverpool </t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>39572</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>KluSTr9s</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>everton</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>AovF1Mia</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>crystal palace</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>48</v>
-      </c>
-      <c r="K6" t="n">
-        <v>481</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>4hy7UG8j</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>45563.45833333334</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">smith j 
-  eng </t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">city ground
-  nottingham </t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>30404</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>UsushcZr</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>nottingham</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>69ZiU2Om</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>fulham</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>48</v>
-      </c>
-      <c r="K7" t="n">
-        <v>481</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>K0JghK0c</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>45563.5625</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">taylor a 
-  eng </t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">molineux stadium
-  wolverhampton </t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>31750</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>j3Azpf5d</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>wolves</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>lId4TMwf</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>liverpool</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>48</v>
-      </c>
-      <c r="K8" t="n">
-        <v>481</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>KnvLwLo4</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>45564.41666666666</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">attwell s 
-  eng </t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">portman road
-  ipswich </t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>29673</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>thqhB2MB</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>ipswich</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>W00wmLO0</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>aston villa</t>
-        </is>
-      </c>
-      <c r="J9" t="n">
-        <v>48</v>
-      </c>
-      <c r="K9" t="n">
-        <v>481</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>SCsTyaGG</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>45564.52083333334</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">kavanagh c 
-  eng </t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">old trafford
-  manchester </t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>75635</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>ppjDR086</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>manchester utd</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>UDg08Ohm</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>tottenham</t>
-        </is>
-      </c>
-      <c r="J10" t="n">
-        <v>48</v>
-      </c>
-      <c r="K10" t="n">
-        <v>481</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
         <is>
           <t>premier league</t>
         </is>

</xml_diff>

<commit_message>
Data. Actualizo predicciones + Entrenamiento USA
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
+++ b/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,45 +507,45 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>r3Wq3yFF</t>
+          <t>ltBAlx0M</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45570.35416666666</v>
+        <v>45571.41666666666</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">hooper s 
+          <t xml:space="preserve">jones r 
   eng </t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">selhurst park
-  london </t>
+          <t xml:space="preserve">villa park
+  birmingham </t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>25486</v>
+        <v>42789</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>AovF1Mia</t>
+          <t>W00wmLO0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>crystal palace</t>
+          <t>aston villa</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>lId4TMwf</t>
+          <t>ppjDR086</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>manchester utd</t>
         </is>
       </c>
       <c r="J2" t="n">
@@ -574,45 +574,45 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>SQM1jbV9</t>
+          <t>nywy5cp3</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45570.45833333334</v>
+        <v>45571.41666666666</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">harrington t 
+          <t xml:space="preserve">kavanagh c 
   eng </t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">emirates stadium
+          <t xml:space="preserve">stamford bridge
   london </t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>60704</v>
+        <v>40341</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>hA1Zm19f</t>
+          <t>4fGZN2oK</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>arsenal</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>WdKOwxDM</t>
+          <t>UsushcZr</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>southampton</t>
+          <t>nottingham</t>
         </is>
       </c>
       <c r="J3" t="n">
@@ -641,45 +641,45 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>bFdtqGNq</t>
+          <t>fsjksfhd</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45570.45833333334</v>
+        <v>45571.52083333334</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">madley a 
+          <t xml:space="preserve">coote d 
   eng </t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">brentford community stadium
-  london </t>
+          <t xml:space="preserve">amex stadium
+  brighton </t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>17250</v>
+        <v>31876</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>xYe7DwID</t>
+          <t>2XrRecc3</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>brentford</t>
+          <t>brighton</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>j3Azpf5d</t>
+          <t>UDg08Ohm</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>wolves</t>
+          <t>tottenham</t>
         </is>
       </c>
       <c r="J4" t="n">
@@ -708,45 +708,40 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>YXAOeg7k</t>
+          <t>OE9k61RO</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45570.45833333334</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bond d 
-  eng </t>
-        </is>
-      </c>
+        <v>45584.35416666666</v>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">king power stadium
-  leicester </t>
+          <t xml:space="preserve">tottenham hotspur stadium
+  london </t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>32261</v>
+        <v>62850</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>KrrdAMyI</t>
+          <t>UDg08Ohm</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>leicester</t>
+          <t>tottenham</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>OtpNdwrc</t>
+          <t>Cxq57r8g</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>bournemouth</t>
+          <t>west ham</t>
         </is>
       </c>
       <c r="J5" t="n">
@@ -775,45 +770,40 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>tbEWgXy2</t>
+          <t>Y5lic6rf</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45570.45833333334</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bankes p 
-  eng </t>
-        </is>
-      </c>
+        <v>45584.45833333334</v>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">etihad stadium
-  manchester </t>
+          <t xml:space="preserve">craven cottage
+  london </t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>55097</v>
+        <v>26600</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Wtn9Stg0</t>
+          <t>69ZiU2Om</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>manchester city</t>
+          <t>fulham</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>69ZiU2Om</t>
+          <t>W00wmLO0</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>fulham</t>
+          <t>aston villa</t>
         </is>
       </c>
       <c r="J6" t="n">
@@ -842,45 +832,40 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>d6dJHzU8</t>
+          <t>tWiaepD6</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>45570.45833333334</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">taylor a 
-  eng </t>
-        </is>
-      </c>
+        <v>45584.45833333334</v>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">london stadium
-  london </t>
+          <t xml:space="preserve">portman road
+  ipswich </t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>62500</v>
+        <v>29673</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Cxq57r8g</t>
+          <t>thqhB2MB</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>west ham</t>
+          <t>ipswich</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>thqhB2MB</t>
+          <t>KluSTr9s</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>ipswich</t>
+          <t>everton</t>
         </is>
       </c>
       <c r="J7" t="n">
@@ -909,45 +894,40 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>l0Zi1FqS</t>
+          <t>UiYgHRZP</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>45570.5625</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pawson c 
-  eng </t>
-        </is>
-      </c>
+        <v>45584.45833333334</v>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">goodison park
-  liverpool </t>
+          <t xml:space="preserve">old trafford
+  manchester </t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>39572</v>
+        <v>75635</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>KluSTr9s</t>
+          <t>ppjDR086</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>everton</t>
+          <t>manchester utd</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>p6ahwuwJ</t>
+          <t>xYe7DwID</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>newcastle</t>
+          <t>brentford</t>
         </is>
       </c>
       <c r="J8" t="n">
@@ -976,45 +956,40 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>ltBAlx0M</t>
+          <t>n9EQB5cm</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45571.41666666666</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">jones r 
-  eng </t>
-        </is>
-      </c>
+        <v>45584.45833333334</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">villa park
-  birmingham </t>
+          <t xml:space="preserve">st  james  park
+  newcastle </t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>42789</v>
+        <v>52305</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>W00wmLO0</t>
+          <t>p6ahwuwJ</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>aston villa</t>
+          <t>newcastle</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>ppjDR086</t>
+          <t>2XrRecc3</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>manchester utd</t>
+          <t>brighton</t>
         </is>
       </c>
       <c r="J9" t="n">
@@ -1043,45 +1018,40 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>nywy5cp3</t>
+          <t>Gl6s8NdC</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>45571.41666666666</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">kavanagh c 
-  eng </t>
-        </is>
-      </c>
+        <v>45584.45833333334</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">stamford bridge
-  london </t>
+          <t xml:space="preserve">st  mary s stadium
+  southampton </t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>40341</v>
+        <v>32384</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>4fGZN2oK</t>
+          <t>WdKOwxDM</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>chelsea</t>
+          <t>southampton</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>UsushcZr</t>
+          <t>KrrdAMyI</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>nottingham</t>
+          <t>leicester</t>
         </is>
       </c>
       <c r="J10" t="n">
@@ -1110,45 +1080,40 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>fsjksfhd</t>
+          <t>ShJjaSDs</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>45571.52083333334</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">coote d 
-  eng </t>
-        </is>
-      </c>
+        <v>45584.5625</v>
+      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">amex stadium
-  brighton </t>
+          <t xml:space="preserve">vitality stadium
+  bournemouth </t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>31876</v>
+        <v>11307</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2XrRecc3</t>
+          <t>OtpNdwrc</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>brighton</t>
+          <t>bournemouth</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>UDg08Ohm</t>
+          <t>hA1Zm19f</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>tottenham</t>
+          <t>arsenal</t>
         </is>
       </c>
       <c r="J11" t="n">
@@ -1177,40 +1142,40 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>OE9k61RO</t>
+          <t>SSZaQ4Ct</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>45584.35416666666</v>
+        <v>45585.41666666666</v>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">tottenham hotspur stadium
-  london </t>
+          <t xml:space="preserve">molineux stadium
+  wolverhampton </t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>62850</v>
+        <v>31750</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>UDg08Ohm</t>
+          <t>j3Azpf5d</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>tottenham</t>
+          <t>wolves</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Cxq57r8g</t>
+          <t>Wtn9Stg0</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>west ham</t>
+          <t>manchester city</t>
         </is>
       </c>
       <c r="J12" t="n">
@@ -1239,40 +1204,40 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Y5lic6rf</t>
+          <t>2ot8gOsJ</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>45584.45833333334</v>
+        <v>45585.52083333334</v>
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">craven cottage
-  london </t>
+          <t xml:space="preserve">anfield
+  liverpool </t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>26600</v>
+        <v>61276</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>69ZiU2Om</t>
+          <t>lId4TMwf</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>fulham</t>
+          <t>liverpool</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>W00wmLO0</t>
+          <t>4fGZN2oK</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>aston villa</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="J13" t="n">
@@ -1293,254 +1258,6 @@
         </is>
       </c>
       <c r="O13" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>tWiaepD6</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>45584.45833333334</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">portman road
-  ipswich </t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>29673</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>thqhB2MB</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>ipswich</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>KluSTr9s</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>everton</t>
-        </is>
-      </c>
-      <c r="J14" t="n">
-        <v>48</v>
-      </c>
-      <c r="K14" t="n">
-        <v>481</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>UiYgHRZP</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>45584.45833333334</v>
-      </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">old trafford
-  manchester </t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>75635</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>ppjDR086</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>manchester utd</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>xYe7DwID</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>brentford</t>
-        </is>
-      </c>
-      <c r="J15" t="n">
-        <v>48</v>
-      </c>
-      <c r="K15" t="n">
-        <v>481</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>n9EQB5cm</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>45584.45833333334</v>
-      </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">st  james  park
-  newcastle </t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>52305</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>p6ahwuwJ</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>newcastle</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>2XrRecc3</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>brighton</t>
-        </is>
-      </c>
-      <c r="J16" t="n">
-        <v>48</v>
-      </c>
-      <c r="K16" t="n">
-        <v>481</v>
-      </c>
-      <c r="L16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>Gl6s8NdC</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>45584.45833333334</v>
-      </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">st  mary s stadium
-  southampton </t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>32384</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>WdKOwxDM</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>southampton</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>KrrdAMyI</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>leicester</t>
-        </is>
-      </c>
-      <c r="J17" t="n">
-        <v>48</v>
-      </c>
-      <c r="K17" t="n">
-        <v>481</v>
-      </c>
-      <c r="L17" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
         <is>
           <t>premier league</t>
         </is>

</xml_diff>

<commit_message>
DATA. Cambio modelo en FRA (x relleno de formaciones) y actualizo predicciones
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
+++ b/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
@@ -513,7 +513,12 @@
       <c r="B2" s="2" t="n">
         <v>45584.35416666666</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">madley a 
+  eng </t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t xml:space="preserve">tottenham hotspur stadium
@@ -575,7 +580,12 @@
       <c r="B3" s="2" t="n">
         <v>45584.45833333334</v>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">england d 
+  eng </t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t xml:space="preserve">craven cottage
@@ -637,7 +647,12 @@
       <c r="B4" s="2" t="n">
         <v>45584.45833333334</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">oliver m 
+  eng </t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
           <t xml:space="preserve">portman road
@@ -699,7 +714,12 @@
       <c r="B5" s="2" t="n">
         <v>45584.45833333334</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">barrott s 
+  eng </t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
           <t xml:space="preserve">old trafford
@@ -761,7 +781,12 @@
       <c r="B6" s="2" t="n">
         <v>45584.45833333334</v>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bankes p 
+  eng </t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
           <t xml:space="preserve">st  james  park
@@ -823,7 +848,12 @@
       <c r="B7" s="2" t="n">
         <v>45584.45833333334</v>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">taylor a 
+  eng </t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
           <t xml:space="preserve">st  mary s stadium
@@ -885,7 +915,12 @@
       <c r="B8" s="2" t="n">
         <v>45584.5625</v>
       </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jones r 
+  eng </t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
           <t xml:space="preserve">vitality stadium
@@ -947,7 +982,12 @@
       <c r="B9" s="2" t="n">
         <v>45585.41666666666</v>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kavanagh c 
+  eng </t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
           <t xml:space="preserve">molineux stadium
@@ -1009,7 +1049,12 @@
       <c r="B10" s="2" t="n">
         <v>45585.52083333334</v>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">brooks j 
+  eng </t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
           <t xml:space="preserve">anfield
@@ -1071,7 +1116,12 @@
       <c r="B11" s="2" t="n">
         <v>45586.66666666666</v>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">robinson t 
+  eng </t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
           <t xml:space="preserve">city ground

</xml_diff>

<commit_message>
DATA. Obtengo predicciones de proximos 15 dias.
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
+++ b/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,199 +507,1238 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>SSZaQ4Ct</t>
+          <t>v5b6XwQN</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45585.41666666666</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">kavanagh c 
-  eng </t>
-        </is>
-      </c>
+        <v>45590.66666666666</v>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king power stadium
+  leicester </t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>32261</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>KrrdAMyI</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>leicester</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>UsushcZr</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>nottingham</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>48</v>
+      </c>
+      <c r="K2" t="n">
+        <v>481</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>ABRGMMB5</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>45591.45833333334</v>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">villa park
+  birmingham </t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>42789</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>W00wmLO0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>aston villa</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>OtpNdwrc</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>bournemouth</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>48</v>
+      </c>
+      <c r="K3" t="n">
+        <v>481</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>rPPOK0tI</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>45591.45833333334</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">brentford community stadium
+  london </t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>17250</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>xYe7DwID</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>brentford</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>thqhB2MB</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>ipswich</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>48</v>
+      </c>
+      <c r="K4" t="n">
+        <v>481</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>viJXIvBU</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>45591.45833333334</v>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">amex stadium
+  brighton </t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>31876</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2XrRecc3</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>brighton</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>j3Azpf5d</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>wolves</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>48</v>
+      </c>
+      <c r="K5" t="n">
+        <v>481</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>zypxSHmo</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>45591.45833333334</v>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">etihad stadium
+  manchester </t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>55097</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Wtn9Stg0</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>manchester city</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>WdKOwxDM</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>southampton</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>48</v>
+      </c>
+      <c r="K6" t="n">
+        <v>481</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>rw5cZaeB</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>45591.5625</v>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">goodison park
+  liverpool </t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>39572</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>KluSTr9s</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>everton</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>69ZiU2Om</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>fulham</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>48</v>
+      </c>
+      <c r="K7" t="n">
+        <v>481</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>EcDtwrdn</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>45592.45833333334</v>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stamford bridge
+  london </t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>40341</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>4fGZN2oK</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>chelsea</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>p6ahwuwJ</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>newcastle</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>48</v>
+      </c>
+      <c r="K8" t="n">
+        <v>481</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>zD1kyMQb</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>45592.45833333334</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">selhurst park
+  london </t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>25486</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>AovF1Mia</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>crystal palace</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>UDg08Ohm</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>tottenham</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>48</v>
+      </c>
+      <c r="K9" t="n">
+        <v>481</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>EJlHkLuh</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>45592.45833333334</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">london stadium
+  london </t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>62500</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Cxq57r8g</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>west ham</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ppjDR086</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>manchester utd</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>48</v>
+      </c>
+      <c r="K10" t="n">
+        <v>481</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>EqY7Orsg</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>45592.5625</v>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">emirates stadium
+  london </t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>60704</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>hA1Zm19f</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>arsenal</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>lId4TMwf</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>liverpool</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>48</v>
+      </c>
+      <c r="K11" t="n">
+        <v>481</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>WIs9mjGL</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>45598.39583333334</v>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">st  james  park
+  newcastle </t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>52305</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>p6ahwuwJ</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>newcastle</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>hA1Zm19f</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>arsenal</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>48</v>
+      </c>
+      <c r="K12" t="n">
+        <v>481</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>MqhPmaA4</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>45598.5</v>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vitality stadium
+  bournemouth </t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>11307</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>OtpNdwrc</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>bournemouth</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Wtn9Stg0</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>manchester city</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>48</v>
+      </c>
+      <c r="K13" t="n">
+        <v>481</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>lb85TUOk</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>45598.5</v>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">portman road
+  ipswich </t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>29673</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>thqhB2MB</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>ipswich</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>KrrdAMyI</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>leicester</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>48</v>
+      </c>
+      <c r="K14" t="n">
+        <v>481</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>rc1ER8g2</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>45598.5</v>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">anfield
+  liverpool </t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>61276</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>lId4TMwf</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>liverpool</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2XrRecc3</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>brighton</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>48</v>
+      </c>
+      <c r="K15" t="n">
+        <v>481</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>21YvrUwq</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>45598.5</v>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">city ground
+  nottingham </t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>30404</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>UsushcZr</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>nottingham</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Cxq57r8g</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>west ham</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>48</v>
+      </c>
+      <c r="K16" t="n">
+        <v>481</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>OGMmt88e</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>45598.5</v>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">st  mary s stadium
+  southampton </t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>32384</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>WdKOwxDM</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>southampton</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>KluSTr9s</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>everton</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>48</v>
+      </c>
+      <c r="K17" t="n">
+        <v>481</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>EJ4unbdE</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>45598.60416666666</v>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
         <is>
           <t xml:space="preserve">molineux stadium
   wolverhampton </t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E18" t="n">
         <v>31750</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>j3Azpf5d</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>wolves</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Wtn9Stg0</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>manchester city</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>48</v>
-      </c>
-      <c r="K2" t="n">
-        <v>481</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>2ot8gOsJ</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>45585.52083333334</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">brooks j 
-  eng </t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">anfield
-  liverpool </t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>61276</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>lId4TMwf</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>liverpool</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>AovF1Mia</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>crystal palace</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>48</v>
+      </c>
+      <c r="K18" t="n">
+        <v>481</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>drzevnw8</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>45599.45833333334</v>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tottenham hotspur stadium
+  london </t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>62850</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>UDg08Ohm</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>tottenham</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>W00wmLO0</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>aston villa</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>48</v>
+      </c>
+      <c r="K19" t="n">
+        <v>481</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>zil0kCo9</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>45599.5625</v>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">old trafford
+  manchester </t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>75635</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>ppjDR086</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>manchester utd</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
         <is>
           <t>4fGZN2oK</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>chelsea</t>
         </is>
       </c>
-      <c r="J3" t="n">
-        <v>48</v>
-      </c>
-      <c r="K3" t="n">
-        <v>481</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>KMCY9qSa</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>45586.66666666666</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">robinson t 
-  eng </t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">city ground
-  nottingham </t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>30404</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>UsushcZr</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>nottingham</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>AovF1Mia</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>crystal palace</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>48</v>
-      </c>
-      <c r="K4" t="n">
-        <v>481</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
+      <c r="J20" t="n">
+        <v>48</v>
+      </c>
+      <c r="K20" t="n">
+        <v>481</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>ratYowuH</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>45600.70833333334</v>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">craven cottage
+  london </t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>26600</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>69ZiU2Om</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>fulham</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>xYe7DwID</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>brentford</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>48</v>
+      </c>
+      <c r="K21" t="n">
+        <v>481</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
         <is>
           <t>premier league</t>
         </is>

</xml_diff>

<commit_message>
DATA. Corro collect pero no actualizo predicciones
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
+++ b/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,7 +513,12 @@
       <c r="B2" s="2" t="n">
         <v>45590.66666666666</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pawson c 
+  eng </t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t xml:space="preserve">king power stadium
@@ -575,7 +580,12 @@
       <c r="B3" s="2" t="n">
         <v>45591.45833333334</v>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">madley a 
+  eng </t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t xml:space="preserve">villa park
@@ -637,7 +647,12 @@
       <c r="B4" s="2" t="n">
         <v>45591.45833333334</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">smith l 
+  eng </t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
           <t xml:space="preserve">brentford community stadium
@@ -699,7 +714,12 @@
       <c r="B5" s="2" t="n">
         <v>45591.45833333334</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">oliver m 
+  eng </t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
           <t xml:space="preserve">amex stadium
@@ -761,7 +781,12 @@
       <c r="B6" s="2" t="n">
         <v>45591.45833333334</v>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">harrington t 
+  eng </t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
           <t xml:space="preserve">etihad stadium
@@ -823,7 +848,12 @@
       <c r="B7" s="2" t="n">
         <v>45591.5625</v>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">brooks j 
+  eng </t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
           <t xml:space="preserve">goodison park
@@ -885,7 +915,12 @@
       <c r="B8" s="2" t="n">
         <v>45592.45833333334</v>
       </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hooper s 
+  eng </t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
           <t xml:space="preserve">stamford bridge
@@ -947,7 +982,12 @@
       <c r="B9" s="2" t="n">
         <v>45592.45833333334</v>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bond d 
+  eng </t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
           <t xml:space="preserve">selhurst park
@@ -1009,7 +1049,12 @@
       <c r="B10" s="2" t="n">
         <v>45592.45833333334</v>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">coote d 
+  eng </t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
           <t xml:space="preserve">london stadium
@@ -1071,7 +1116,12 @@
       <c r="B11" s="2" t="n">
         <v>45592.5625</v>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">taylor a 
+  eng </t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
           <t xml:space="preserve">emirates stadium
@@ -1119,626 +1169,6 @@
         </is>
       </c>
       <c r="O11" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>WIs9mjGL</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>45598.39583333334</v>
-      </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">st  james  park
-  newcastle </t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>52305</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>p6ahwuwJ</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>newcastle</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>hA1Zm19f</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>arsenal</t>
-        </is>
-      </c>
-      <c r="J12" t="n">
-        <v>48</v>
-      </c>
-      <c r="K12" t="n">
-        <v>481</v>
-      </c>
-      <c r="L12" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>MqhPmaA4</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>45598.5</v>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">vitality stadium
-  bournemouth </t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>11307</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>OtpNdwrc</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>bournemouth</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Wtn9Stg0</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>manchester city</t>
-        </is>
-      </c>
-      <c r="J13" t="n">
-        <v>48</v>
-      </c>
-      <c r="K13" t="n">
-        <v>481</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>lb85TUOk</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>45598.5</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">portman road
-  ipswich </t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>29673</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>thqhB2MB</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>ipswich</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>KrrdAMyI</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>leicester</t>
-        </is>
-      </c>
-      <c r="J14" t="n">
-        <v>48</v>
-      </c>
-      <c r="K14" t="n">
-        <v>481</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>rc1ER8g2</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>45598.5</v>
-      </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">anfield
-  liverpool </t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>61276</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>lId4TMwf</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>liverpool</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>2XrRecc3</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>brighton</t>
-        </is>
-      </c>
-      <c r="J15" t="n">
-        <v>48</v>
-      </c>
-      <c r="K15" t="n">
-        <v>481</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>21YvrUwq</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>45598.5</v>
-      </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">city ground
-  nottingham </t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>30404</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>UsushcZr</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>nottingham</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Cxq57r8g</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>west ham</t>
-        </is>
-      </c>
-      <c r="J16" t="n">
-        <v>48</v>
-      </c>
-      <c r="K16" t="n">
-        <v>481</v>
-      </c>
-      <c r="L16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>OGMmt88e</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>45598.5</v>
-      </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">st  mary s stadium
-  southampton </t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>32384</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>WdKOwxDM</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>southampton</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>KluSTr9s</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>everton</t>
-        </is>
-      </c>
-      <c r="J17" t="n">
-        <v>48</v>
-      </c>
-      <c r="K17" t="n">
-        <v>481</v>
-      </c>
-      <c r="L17" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>EJ4unbdE</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>45598.60416666666</v>
-      </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">molineux stadium
-  wolverhampton </t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>31750</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>j3Azpf5d</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>wolves</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>AovF1Mia</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>crystal palace</t>
-        </is>
-      </c>
-      <c r="J18" t="n">
-        <v>48</v>
-      </c>
-      <c r="K18" t="n">
-        <v>481</v>
-      </c>
-      <c r="L18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>drzevnw8</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="n">
-        <v>45599.45833333334</v>
-      </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tottenham hotspur stadium
-  london </t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>62850</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>UDg08Ohm</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>tottenham</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>W00wmLO0</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>aston villa</t>
-        </is>
-      </c>
-      <c r="J19" t="n">
-        <v>48</v>
-      </c>
-      <c r="K19" t="n">
-        <v>481</v>
-      </c>
-      <c r="L19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>zil0kCo9</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="n">
-        <v>45599.5625</v>
-      </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">old trafford
-  manchester </t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>75635</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>ppjDR086</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>manchester utd</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>4fGZN2oK</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>chelsea</t>
-        </is>
-      </c>
-      <c r="J20" t="n">
-        <v>48</v>
-      </c>
-      <c r="K20" t="n">
-        <v>481</v>
-      </c>
-      <c r="L20" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>ratYowuH</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>45600.70833333334</v>
-      </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">craven cottage
-  london </t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>26600</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>69ZiU2Om</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>fulham</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>xYe7DwID</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>brentford</t>
-        </is>
-      </c>
-      <c r="J21" t="n">
-        <v>48</v>
-      </c>
-      <c r="K21" t="n">
-        <v>481</v>
-      </c>
-      <c r="L21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
         <is>
           <t>premier league</t>
         </is>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones del fin de semana x missing y cuotas.
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
+++ b/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1169,626 +1169,6 @@
         </is>
       </c>
       <c r="O11" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>nX2mpxRQ</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>45605.5</v>
-      </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">brentford community stadium
-  london </t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>17250</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>xYe7DwID</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>brentford</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>OtpNdwrc</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>bournemouth</t>
-        </is>
-      </c>
-      <c r="J12" t="n">
-        <v>48</v>
-      </c>
-      <c r="K12" t="n">
-        <v>481</v>
-      </c>
-      <c r="L12" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>YTzyyYmD</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>45605.5</v>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">selhurst park
-  london </t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>25486</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>AovF1Mia</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>crystal palace</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>69ZiU2Om</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>fulham</t>
-        </is>
-      </c>
-      <c r="J13" t="n">
-        <v>48</v>
-      </c>
-      <c r="K13" t="n">
-        <v>481</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>K0RAmBXI</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>45605.5</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">london stadium
-  london </t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>62500</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Cxq57r8g</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>west ham</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>KluSTr9s</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>everton</t>
-        </is>
-      </c>
-      <c r="J14" t="n">
-        <v>48</v>
-      </c>
-      <c r="K14" t="n">
-        <v>481</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>0d4cBEPP</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>45605.5</v>
-      </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">molineux stadium
-  wolverhampton </t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>31750</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>j3Azpf5d</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>wolves</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>WdKOwxDM</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>southampton</t>
-        </is>
-      </c>
-      <c r="J15" t="n">
-        <v>48</v>
-      </c>
-      <c r="K15" t="n">
-        <v>481</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>6HqKvGll</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>45605.60416666666</v>
-      </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">amex stadium
-  brighton </t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>31876</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>2XrRecc3</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>brighton</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Wtn9Stg0</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>manchester city</t>
-        </is>
-      </c>
-      <c r="J16" t="n">
-        <v>48</v>
-      </c>
-      <c r="K16" t="n">
-        <v>481</v>
-      </c>
-      <c r="L16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>0zTMbytK</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>45605.70833333334</v>
-      </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">anfield
-  liverpool </t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>61276</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>lId4TMwf</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>liverpool</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>W00wmLO0</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>aston villa</t>
-        </is>
-      </c>
-      <c r="J17" t="n">
-        <v>48</v>
-      </c>
-      <c r="K17" t="n">
-        <v>481</v>
-      </c>
-      <c r="L17" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>KK9ggF3s</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>45606.45833333334</v>
-      </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">old trafford
-  manchester </t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>75635</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>ppjDR086</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>manchester utd</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>KrrdAMyI</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>leicester</t>
-        </is>
-      </c>
-      <c r="J18" t="n">
-        <v>48</v>
-      </c>
-      <c r="K18" t="n">
-        <v>481</v>
-      </c>
-      <c r="L18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>hY71igYg</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="n">
-        <v>45606.45833333334</v>
-      </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">city ground
-  nottingham </t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>30404</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>UsushcZr</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>nottingham</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>p6ahwuwJ</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>newcastle</t>
-        </is>
-      </c>
-      <c r="J19" t="n">
-        <v>48</v>
-      </c>
-      <c r="K19" t="n">
-        <v>481</v>
-      </c>
-      <c r="L19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>CzO2kX26</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="n">
-        <v>45606.45833333334</v>
-      </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tottenham hotspur stadium
-  london </t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>62850</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>UDg08Ohm</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>tottenham</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>thqhB2MB</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>ipswich</t>
-        </is>
-      </c>
-      <c r="J20" t="n">
-        <v>48</v>
-      </c>
-      <c r="K20" t="n">
-        <v>481</v>
-      </c>
-      <c r="L20" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>CEnSxfJ0</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>45606.5625</v>
-      </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">stamford bridge
-  london </t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>40341</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>4fGZN2oK</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>chelsea</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>hA1Zm19f</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>arsenal</t>
-        </is>
-      </c>
-      <c r="J21" t="n">
-        <v>48</v>
-      </c>
-      <c r="K21" t="n">
-        <v>481</v>
-      </c>
-      <c r="L21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" t="n">
-        <v>20242025</v>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
         <is>
           <t>premier league</t>
         </is>

</xml_diff>

<commit_message>
DATA. Comienzo a reeentrenar modelos con missing + actualizo predicciones segun nuevos modelos
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
+++ b/data/england/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1049,7 +1049,12 @@
       <c r="B10" s="2" t="n">
         <v>45606.45833333334</v>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">england d 
+  eng </t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
           <t xml:space="preserve">tottenham hotspur stadium
@@ -1164,6 +1169,440 @@
         </is>
       </c>
       <c r="O11" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>EubK3NNG</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>45619.39583333334</v>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king power stadium
+  leicester </t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>32261</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>KrrdAMyI</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>leicester</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>4fGZN2oK</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>chelsea</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>48</v>
+      </c>
+      <c r="K12" t="n">
+        <v>481</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>Cl3y4WHa</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>45619.5</v>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">emirates stadium
+  london </t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>60704</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>hA1Zm19f</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>arsenal</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>UsushcZr</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>nottingham</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>48</v>
+      </c>
+      <c r="K13" t="n">
+        <v>481</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>p21q2AnC</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>45619.5</v>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">villa park
+  birmingham </t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>42789</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>W00wmLO0</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>aston villa</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>AovF1Mia</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>crystal palace</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>48</v>
+      </c>
+      <c r="K14" t="n">
+        <v>481</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>WveT5hmm</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>45619.5</v>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vitality stadium
+  bournemouth </t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>11307</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>OtpNdwrc</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>bournemouth</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2XrRecc3</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>brighton</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>48</v>
+      </c>
+      <c r="K15" t="n">
+        <v>481</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>v3JHq2Wp</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>45619.5</v>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">goodison park
+  liverpool </t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>39572</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>KluSTr9s</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>everton</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>xYe7DwID</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>brentford</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>48</v>
+      </c>
+      <c r="K16" t="n">
+        <v>481</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>69B375Oi</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>45619.5</v>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">craven cottage
+  london </t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>29589</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>69ZiU2Om</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>fulham</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>j3Azpf5d</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>wolves</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>48</v>
+      </c>
+      <c r="K17" t="n">
+        <v>481</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>A7iT11hT</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>45619.60416666666</v>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">etihad stadium
+  manchester </t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>55097</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Wtn9Stg0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>manchester city</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>UDg08Ohm</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>tottenham</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>48</v>
+      </c>
+      <c r="K18" t="n">
+        <v>481</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
         <is>
           <t>premier league</t>
         </is>

</xml_diff>